<commit_message>
Add Verified, Asset, Target, Vuln columns to Security Issues tab
Security Issues sheet now includes four additional columns:
  Verified – default 'Y' for all findings
  Asset    – device name (switch label or array name)
  Target   – Object / Interface + (config line) combined
  Vuln     – 'SAN - <Category>' for each finding

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/san/sample-san_analysis.xlsx
+++ b/san/sample-san_analysis.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCI DSS Mapping" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Security Issues'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Security Issues'!$A$1:$N$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -124,6 +124,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="14"/>
     </font>
@@ -145,7 +151,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -190,6 +196,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -239,7 +250,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -329,6 +340,9 @@
     <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -338,28 +352,28 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -748,7 +762,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-15 15:36:03    Switches: swd77 Domain 1; swd77 Domain 2    Array: ZZZZZ01p-mp HPE Alletra Storage</t>
+          <t>Generated: 2026-06-15 22:52:00    Switches: swd77 Domain 1; swd77 Domain 2    Array: ZZZZZ01p-mp HPE Alletra Storage</t>
         </is>
       </c>
     </row>
@@ -2927,7 +2941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2940,6 +2954,10 @@
     <col width="60" customWidth="1" min="8" max="8"/>
     <col width="60" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -2993,6 +3011,26 @@
           <t>Details</t>
         </is>
       </c>
+      <c r="K1" s="9" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="L1" s="9" t="inlineStr">
+        <is>
+          <t>Asset</t>
+        </is>
+      </c>
+      <c r="M1" s="9" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="N1" s="9" t="inlineStr">
+        <is>
+          <t>Vuln</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="29" t="n">
@@ -3043,6 +3081,26 @@
           <t>configShow line 22</t>
         </is>
       </c>
+      <c r="K2" s="33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L2" s="20" t="inlineStr">
+        <is>
+          <t>swd77 (Domain 1)</t>
+        </is>
+      </c>
+      <c r="M2" s="20" t="inlineStr">
+        <is>
+          <t>auth.policy: 0 (off) (22)</t>
+        </is>
+      </c>
+      <c r="N2" s="20" t="inlineStr">
+        <is>
+          <t>SAN - FC Authentication Policy Disabled</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="40" customHeight="1">
       <c r="A3" s="15" t="n">
@@ -3063,17 +3121,17 @@
           <t>defzone: allaccess</t>
         </is>
       </c>
-      <c r="E3" s="33" t="inlineStr">
+      <c r="E3" s="34" t="inlineStr">
         <is>
           <t>359</t>
         </is>
       </c>
-      <c r="F3" s="34" t="inlineStr">
+      <c r="F3" s="35" t="inlineStr">
         <is>
           <t>CIS 12.2 · CIS 13.4</t>
         </is>
       </c>
-      <c r="G3" s="35" t="inlineStr">
+      <c r="G3" s="36" t="inlineStr">
         <is>
           <t>PCI 1.2.4 · PCI 1.3.2</t>
         </is>
@@ -3091,6 +3149,26 @@
       <c r="J3" s="21" t="inlineStr">
         <is>
           <t>configShow line 359</t>
+        </is>
+      </c>
+      <c r="K3" s="33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L3" s="21" t="inlineStr">
+        <is>
+          <t>swd77 (Domain 1)</t>
+        </is>
+      </c>
+      <c r="M3" s="21" t="inlineStr">
+        <is>
+          <t>defzone: allaccess (359)</t>
+        </is>
+      </c>
+      <c r="N3" s="21" t="inlineStr">
+        <is>
+          <t>SAN - Default Zone Allows All Access</t>
         </is>
       </c>
     </row>
@@ -3143,6 +3221,26 @@
           <t>configShow line 22</t>
         </is>
       </c>
+      <c r="K4" s="33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L4" s="20" t="inlineStr">
+        <is>
+          <t>swd77 (Domain 2)</t>
+        </is>
+      </c>
+      <c r="M4" s="20" t="inlineStr">
+        <is>
+          <t>auth.policy: 0 (off) (22)</t>
+        </is>
+      </c>
+      <c r="N4" s="20" t="inlineStr">
+        <is>
+          <t>SAN - FC Authentication Policy Disabled</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="15" t="n">
@@ -3163,17 +3261,17 @@
           <t>defzone: allaccess</t>
         </is>
       </c>
-      <c r="E5" s="33" t="inlineStr">
+      <c r="E5" s="34" t="inlineStr">
         <is>
           <t>357</t>
         </is>
       </c>
-      <c r="F5" s="34" t="inlineStr">
+      <c r="F5" s="35" t="inlineStr">
         <is>
           <t>CIS 12.2 · CIS 13.4</t>
         </is>
       </c>
-      <c r="G5" s="35" t="inlineStr">
+      <c r="G5" s="36" t="inlineStr">
         <is>
           <t>PCI 1.2.4 · PCI 1.3.2</t>
         </is>
@@ -3191,6 +3289,26 @@
       <c r="J5" s="21" t="inlineStr">
         <is>
           <t>configShow line 357</t>
+        </is>
+      </c>
+      <c r="K5" s="33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L5" s="21" t="inlineStr">
+        <is>
+          <t>swd77 (Domain 2)</t>
+        </is>
+      </c>
+      <c r="M5" s="21" t="inlineStr">
+        <is>
+          <t>defzone: allaccess (357)</t>
+        </is>
+      </c>
+      <c r="N5" s="21" t="inlineStr">
+        <is>
+          <t>SAN - Default Zone Allows All Access</t>
         </is>
       </c>
     </row>
@@ -3239,6 +3357,26 @@
           <t>showhost -chap: ESX02, ESX04, ESX05, ESX06, ESX07</t>
         </is>
       </c>
+      <c r="K6" s="33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L6" s="20" t="inlineStr">
+        <is>
+          <t>ZZZZZ01p-mp</t>
+        </is>
+      </c>
+      <c r="M6" s="20" t="inlineStr">
+        <is>
+          <t>5 host(s) without CHAP</t>
+        </is>
+      </c>
+      <c r="N6" s="20" t="inlineStr">
+        <is>
+          <t>SAN - No CHAP on Storage Hosts</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="15" t="n">
@@ -3259,13 +3397,13 @@
           <t>commands: showpasswordpolicy, showsnmp, showsyslog, showaudit, showtime</t>
         </is>
       </c>
-      <c r="E7" s="33" t="inlineStr"/>
-      <c r="F7" s="34" t="inlineStr">
+      <c r="E7" s="34" t="inlineStr"/>
+      <c r="F7" s="35" t="inlineStr">
         <is>
           <t>CIS 4.2 · CIS 8.2</t>
         </is>
       </c>
-      <c r="G7" s="35" t="inlineStr">
+      <c r="G7" s="36" t="inlineStr">
         <is>
           <t>PCI 2.2.1 · PCI 10.5.4</t>
         </is>
@@ -3283,6 +3421,26 @@
       <c r="J7" s="21" t="inlineStr">
         <is>
           <t>Invalid on this firmware: showpasswordpolicy, showsnmp, showsyslog, showaudit, showtime</t>
+        </is>
+      </c>
+      <c r="K7" s="33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L7" s="21" t="inlineStr">
+        <is>
+          <t>ZZZZZ01p-mp</t>
+        </is>
+      </c>
+      <c r="M7" s="21" t="inlineStr">
+        <is>
+          <t>commands: showpasswordpolicy, showsnmp, showsyslog, showaudit, showtime</t>
+        </is>
+      </c>
+      <c r="N7" s="21" t="inlineStr">
+        <is>
+          <t>SAN - Security Baseline Not Verifiable</t>
         </is>
       </c>
     </row>
@@ -3331,6 +3489,26 @@
           <t>showsshkey: No SSH key found</t>
         </is>
       </c>
+      <c r="K8" s="33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L8" s="20" t="inlineStr">
+        <is>
+          <t>ZZZZZ01p-mp</t>
+        </is>
+      </c>
+      <c r="M8" s="20" t="inlineStr">
+        <is>
+          <t>showsshkey: No SSH key found</t>
+        </is>
+      </c>
+      <c r="N8" s="20" t="inlineStr">
+        <is>
+          <t>SAN - No SSH Keys Configured</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="15" t="n">
@@ -3351,13 +3529,13 @@
           <t>Volume Set: DevTest1</t>
         </is>
       </c>
-      <c r="E9" s="33" t="inlineStr"/>
-      <c r="F9" s="34" t="inlineStr">
+      <c r="E9" s="34" t="inlineStr"/>
+      <c r="F9" s="35" t="inlineStr">
         <is>
           <t>CIS 11.1 · CIS 11.2</t>
         </is>
       </c>
-      <c r="G9" s="35" t="inlineStr"/>
+      <c r="G9" s="36" t="inlineStr"/>
       <c r="H9" s="21" t="inlineStr">
         <is>
           <t>Volume set 'DevTest1' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
@@ -3371,6 +3549,26 @@
       <c r="J9" s="21" t="inlineStr">
         <is>
           <t>Protection: Local Snapshots | Replication: None</t>
+        </is>
+      </c>
+      <c r="K9" s="33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L9" s="21" t="inlineStr">
+        <is>
+          <t>hai01p-mp</t>
+        </is>
+      </c>
+      <c r="M9" s="21" t="inlineStr">
+        <is>
+          <t>Volume Set: DevTest1</t>
+        </is>
+      </c>
+      <c r="N9" s="21" t="inlineStr">
+        <is>
+          <t>SAN - No Volume Replication Configured</t>
         </is>
       </c>
     </row>
@@ -3415,6 +3613,26 @@
           <t>Protection: Local Snapshots | Replication: None</t>
         </is>
       </c>
+      <c r="K10" s="33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L10" s="20" t="inlineStr">
+        <is>
+          <t>hai01p-mp</t>
+        </is>
+      </c>
+      <c r="M10" s="20" t="inlineStr">
+        <is>
+          <t>Volume Set: Infrastructure1</t>
+        </is>
+      </c>
+      <c r="N10" s="20" t="inlineStr">
+        <is>
+          <t>SAN - No Volume Replication Configured</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="15" t="n">
@@ -3435,13 +3653,13 @@
           <t>Volume Set: Infrastructure2</t>
         </is>
       </c>
-      <c r="E11" s="33" t="inlineStr"/>
-      <c r="F11" s="34" t="inlineStr">
+      <c r="E11" s="34" t="inlineStr"/>
+      <c r="F11" s="35" t="inlineStr">
         <is>
           <t>CIS 11.1 · CIS 11.2</t>
         </is>
       </c>
-      <c r="G11" s="35" t="inlineStr"/>
+      <c r="G11" s="36" t="inlineStr"/>
       <c r="H11" s="21" t="inlineStr">
         <is>
           <t>Volume set 'Infrastructure2' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
@@ -3455,6 +3673,26 @@
       <c r="J11" s="21" t="inlineStr">
         <is>
           <t>Protection: Local Snapshots | Replication: None</t>
+        </is>
+      </c>
+      <c r="K11" s="33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L11" s="21" t="inlineStr">
+        <is>
+          <t>hai01p-mp</t>
+        </is>
+      </c>
+      <c r="M11" s="21" t="inlineStr">
+        <is>
+          <t>Volume Set: Infrastructure2</t>
+        </is>
+      </c>
+      <c r="N11" s="21" t="inlineStr">
+        <is>
+          <t>SAN - No Volume Replication Configured</t>
         </is>
       </c>
     </row>
@@ -3499,6 +3737,26 @@
           <t>Protection: Local Snapshots | Replication: None</t>
         </is>
       </c>
+      <c r="K12" s="33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L12" s="20" t="inlineStr">
+        <is>
+          <t>hai01p-mp</t>
+        </is>
+      </c>
+      <c r="M12" s="20" t="inlineStr">
+        <is>
+          <t>Volume Set: Production1</t>
+        </is>
+      </c>
+      <c r="N12" s="20" t="inlineStr">
+        <is>
+          <t>SAN - No Volume Replication Configured</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="40" customHeight="1">
       <c r="A13" s="15" t="n">
@@ -3519,13 +3777,13 @@
           <t>Volume Set: Production2</t>
         </is>
       </c>
-      <c r="E13" s="33" t="inlineStr"/>
-      <c r="F13" s="34" t="inlineStr">
+      <c r="E13" s="34" t="inlineStr"/>
+      <c r="F13" s="35" t="inlineStr">
         <is>
           <t>CIS 11.1 · CIS 11.2</t>
         </is>
       </c>
-      <c r="G13" s="35" t="inlineStr"/>
+      <c r="G13" s="36" t="inlineStr"/>
       <c r="H13" s="21" t="inlineStr">
         <is>
           <t>Volume set 'Production2' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
@@ -3539,6 +3797,26 @@
       <c r="J13" s="21" t="inlineStr">
         <is>
           <t>Protection: Local Snapshots | Replication: None</t>
+        </is>
+      </c>
+      <c r="K13" s="33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L13" s="21" t="inlineStr">
+        <is>
+          <t>hai01p-mp</t>
+        </is>
+      </c>
+      <c r="M13" s="21" t="inlineStr">
+        <is>
+          <t>Volume Set: Production2</t>
+        </is>
+      </c>
+      <c r="N13" s="21" t="inlineStr">
+        <is>
+          <t>SAN - No Volume Replication Configured</t>
         </is>
       </c>
     </row>
@@ -3591,6 +3869,26 @@
           <t>configShow line 377</t>
         </is>
       </c>
+      <c r="K14" s="33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L14" s="20" t="inlineStr">
+        <is>
+          <t>swd77 (Domain 1)</t>
+        </is>
+      </c>
+      <c r="M14" s="20" t="inlineStr">
+        <is>
+          <t>[Banner] section empty (377)</t>
+        </is>
+      </c>
+      <c r="N14" s="20" t="inlineStr">
+        <is>
+          <t>SAN - No Login Banner Configured</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="40" customHeight="1">
       <c r="A15" s="15" t="n">
@@ -3611,17 +3909,17 @@
           <t>4 orphaned zone(s)</t>
         </is>
       </c>
-      <c r="E15" s="33" t="inlineStr">
+      <c r="E15" s="34" t="inlineStr">
         <is>
           <t>419</t>
         </is>
       </c>
-      <c r="F15" s="34" t="inlineStr">
+      <c r="F15" s="35" t="inlineStr">
         <is>
           <t>CIS 12.2</t>
         </is>
       </c>
-      <c r="G15" s="35" t="inlineStr"/>
+      <c r="G15" s="36" t="inlineStr"/>
       <c r="H15" s="21" t="inlineStr">
         <is>
           <t>4 zone(s) are defined but not included in any active zone configuration (cfg): z_EXCHANGE2_EVA2_A; z_SQLPROD2_EVA2_A; z_SQLPROD_EVA2_A; z_SQLTEST_EVA2_A. These may represent decommissioned hosts or legacy storage (e.g., EVA2 arrays) removed without zone cleanup. Stale zones inflate configuration and may be accidentally re-activated.</t>
@@ -3635,6 +3933,26 @@
       <c r="J15" s="21" t="inlineStr">
         <is>
           <t>z_EXCHANGE2_EVA2_A; z_SQLPROD2_EVA2_A; z_SQLPROD_EVA2_A; z_SQLTEST_EVA2_A</t>
+        </is>
+      </c>
+      <c r="K15" s="33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L15" s="21" t="inlineStr">
+        <is>
+          <t>swd77 (Domain 1)</t>
+        </is>
+      </c>
+      <c r="M15" s="21" t="inlineStr">
+        <is>
+          <t>4 orphaned zone(s) (419)</t>
+        </is>
+      </c>
+      <c r="N15" s="21" t="inlineStr">
+        <is>
+          <t>SAN - Stale Zone Definitions</t>
         </is>
       </c>
     </row>
@@ -3687,6 +4005,26 @@
           <t>configShow line 375</t>
         </is>
       </c>
+      <c r="K16" s="33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L16" s="20" t="inlineStr">
+        <is>
+          <t>swd77 (Domain 2)</t>
+        </is>
+      </c>
+      <c r="M16" s="20" t="inlineStr">
+        <is>
+          <t>[Banner] section empty (375)</t>
+        </is>
+      </c>
+      <c r="N16" s="20" t="inlineStr">
+        <is>
+          <t>SAN - No Login Banner Configured</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="40" customHeight="1">
       <c r="A17" s="15" t="n">
@@ -3707,17 +4045,17 @@
           <t>5 orphaned zone(s)</t>
         </is>
       </c>
-      <c r="E17" s="33" t="inlineStr">
+      <c r="E17" s="34" t="inlineStr">
         <is>
           <t>417</t>
         </is>
       </c>
-      <c r="F17" s="34" t="inlineStr">
+      <c r="F17" s="35" t="inlineStr">
         <is>
           <t>CIS 12.2</t>
         </is>
       </c>
-      <c r="G17" s="35" t="inlineStr"/>
+      <c r="G17" s="36" t="inlineStr"/>
       <c r="H17" s="21" t="inlineStr">
         <is>
           <t>5 zone(s) are defined but not included in any active zone configuration (cfg): z_EXCHANGE2_EVA2_B; z_SQLPROD2_EVA2_B; z_SQLPROD_EVA2_B; z_SQLTEST2_EVA_B; z_SQLTEST_EVA_B. These may represent decommissioned hosts or legacy storage (e.g., EVA2 arrays) removed without zone cleanup. Stale zones inflate configuration and may be accidentally re-activated.</t>
@@ -3731,6 +4069,26 @@
       <c r="J17" s="21" t="inlineStr">
         <is>
           <t>z_EXCHANGE2_EVA2_B; z_SQLPROD2_EVA2_B; z_SQLPROD_EVA2_B; z_SQLTEST2_EVA_B; z_SQLTEST_EVA_B</t>
+        </is>
+      </c>
+      <c r="K17" s="33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L17" s="21" t="inlineStr">
+        <is>
+          <t>swd77 (Domain 2)</t>
+        </is>
+      </c>
+      <c r="M17" s="21" t="inlineStr">
+        <is>
+          <t>5 orphaned zone(s) (417)</t>
+        </is>
+      </c>
+      <c r="N17" s="21" t="inlineStr">
+        <is>
+          <t>SAN - Stale Zone Definitions</t>
         </is>
       </c>
     </row>
@@ -3775,6 +4133,26 @@
           <t>Ports in loss_sync: 0:3:2, 0:3:4, 1:3:2, 1:3:4</t>
         </is>
       </c>
+      <c r="K18" s="33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L18" s="20" t="inlineStr">
+        <is>
+          <t>ZZZZZ01p-mp</t>
+        </is>
+      </c>
+      <c r="M18" s="20" t="inlineStr">
+        <is>
+          <t>loss_sync: 0:3:2, 0:3:4, 1:3:2, 1:3:4</t>
+        </is>
+      </c>
+      <c r="N18" s="20" t="inlineStr">
+        <is>
+          <t>SAN - Degraded FC Ports</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="40" customHeight="1">
       <c r="A19" s="15" t="n">
@@ -3795,13 +4173,13 @@
           <t>WSAPI: Enabled / Active on HTTPS 443</t>
         </is>
       </c>
-      <c r="E19" s="33" t="inlineStr"/>
-      <c r="F19" s="34" t="inlineStr">
+      <c r="E19" s="34" t="inlineStr"/>
+      <c r="F19" s="35" t="inlineStr">
         <is>
           <t>CIS 4.8 · CIS 12.3</t>
         </is>
       </c>
-      <c r="G19" s="35" t="inlineStr">
+      <c r="G19" s="36" t="inlineStr">
         <is>
           <t>PCI 2.2.4</t>
         </is>
@@ -3819,6 +4197,26 @@
       <c r="J19" s="21" t="inlineStr">
         <is>
           <t>WSAPI: Enabled / Active, HTTPS 443</t>
+        </is>
+      </c>
+      <c r="K19" s="33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L19" s="21" t="inlineStr">
+        <is>
+          <t>ZZZZZ01p-mp</t>
+        </is>
+      </c>
+      <c r="M19" s="21" t="inlineStr">
+        <is>
+          <t>WSAPI: Enabled / Active on HTTPS 443</t>
+        </is>
+      </c>
+      <c r="N19" s="21" t="inlineStr">
+        <is>
+          <t>SAN - REST API Exposed</t>
         </is>
       </c>
     </row>
@@ -3859,6 +4257,26 @@
         </is>
       </c>
       <c r="J20" s="20" t="inlineStr"/>
+      <c r="K20" s="33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L20" s="20" t="inlineStr">
+        <is>
+          <t>swd77 (Domain 1)</t>
+        </is>
+      </c>
+      <c r="M20" s="20" t="inlineStr">
+        <is>
+          <t>maps.activePolicy: dflt_base_policy</t>
+        </is>
+      </c>
+      <c r="N20" s="20" t="inlineStr">
+        <is>
+          <t>SAN - Default MAPS Monitoring Policy</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="40" customHeight="1">
       <c r="A21" s="15" t="n">
@@ -3879,13 +4297,13 @@
           <t>maps.activePolicy: dflt_base_policy</t>
         </is>
       </c>
-      <c r="E21" s="33" t="inlineStr"/>
-      <c r="F21" s="34" t="inlineStr">
+      <c r="E21" s="34" t="inlineStr"/>
+      <c r="F21" s="35" t="inlineStr">
         <is>
           <t>CIS 8.2</t>
         </is>
       </c>
-      <c r="G21" s="35" t="inlineStr"/>
+      <c r="G21" s="36" t="inlineStr"/>
       <c r="H21" s="21" t="inlineStr">
         <is>
           <t>MAPS is using the default policy 'dflt_base_policy' rather than a customized environment-specific policy. Default thresholds may not match this fabric's traffic patterns, causing missed alerts or excessive noise.</t>
@@ -3897,6 +4315,26 @@
         </is>
       </c>
       <c r="J21" s="21" t="inlineStr"/>
+      <c r="K21" s="33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L21" s="21" t="inlineStr">
+        <is>
+          <t>swd77 (Domain 2)</t>
+        </is>
+      </c>
+      <c r="M21" s="21" t="inlineStr">
+        <is>
+          <t>maps.activePolicy: dflt_base_policy</t>
+        </is>
+      </c>
+      <c r="N21" s="21" t="inlineStr">
+        <is>
+          <t>SAN - Default MAPS Monitoring Policy</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="40" customHeight="1">
       <c r="A22" s="29" t="n">
@@ -3939,9 +4377,29 @@
           <t>naa.60002ac0000000000000002b0002e9bd; naa.60002ac0000000000000002c0002e9bd; naa.60002ac0000000000000002e0002e9bd; naa.60002ac000000000000000130002e9bd; naa.60002ac0000000000000002d0002e9bd</t>
         </is>
       </c>
+      <c r="K22" s="33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L22" s="20" t="inlineStr">
+        <is>
+          <t>VMware ESXi</t>
+        </is>
+      </c>
+      <c r="M22" s="20" t="inlineStr">
+        <is>
+          <t>5 FC disk(s)</t>
+        </is>
+      </c>
+      <c r="N22" s="20" t="inlineStr">
+        <is>
+          <t>SAN - Perennially Reserved Not Configured</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
+  <autoFilter ref="A1:N1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3964,7 +4422,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="36" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>CIS Controls v8 — Finding Cross-Reference</t>
         </is>
@@ -3978,39 +4436,39 @@
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="37" t="inlineStr">
+      <c r="A4" s="38" t="inlineStr">
         <is>
           <t>CIS 3.10 — Encrypt Sensitive Data in Transit</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="38" t="inlineStr">
+      <c r="A5" s="39" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B5" s="38" t="inlineStr">
+      <c r="B5" s="39" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C5" s="38" t="inlineStr">
+      <c r="C5" s="39" t="inlineStr">
         <is>
           <t>Object / Interface</t>
         </is>
       </c>
-      <c r="D5" s="38" t="inlineStr">
+      <c r="D5" s="39" t="inlineStr">
         <is>
           <t>Config Line</t>
         </is>
       </c>
-      <c r="E5" s="38" t="inlineStr">
+      <c r="E5" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F5" s="38" t="inlineStr">
+      <c r="F5" s="39" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
@@ -4032,7 +4490,7 @@
           <t>5 host(s) without CHAP</t>
         </is>
       </c>
-      <c r="D6" s="39" t="inlineStr"/>
+      <c r="D6" s="40" t="inlineStr"/>
       <c r="E6" s="20" t="inlineStr">
         <is>
           <t>No CHAP authentication is configured for 5 ESX host(s): ESX02, ESX04, ESX05, ESX06, ESX07. Both Initiator CHAP and Target CHAP show '--' in 'showhost -chap'. Without CHAP, any host presenting the correct WWN can authenticate to the array. In a compromised or miscabled environment this allows unauthorized LUN access.</t>
@@ -4060,7 +4518,7 @@
           <t>showsshkey: No SSH key found</t>
         </is>
       </c>
-      <c r="D7" s="40" t="inlineStr"/>
+      <c r="D7" s="41" t="inlineStr"/>
       <c r="E7" s="21" t="inlineStr">
         <is>
           <t>No SSH public keys are configured on the Alletra MP. Administrative access relies exclusively on password authentication. Password-only authentication is weaker than key-based auth and does not meet PCI DSS requirements for strong cryptographic access controls.</t>
@@ -4073,39 +4531,39 @@
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="37" t="inlineStr">
+      <c r="A9" s="38" t="inlineStr">
         <is>
           <t>CIS 4.2 — Secure Configuration Process for Network Infrastructure</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="38" t="inlineStr">
+      <c r="A10" s="39" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B10" s="38" t="inlineStr">
+      <c r="B10" s="39" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C10" s="38" t="inlineStr">
+      <c r="C10" s="39" t="inlineStr">
         <is>
           <t>Object / Interface</t>
         </is>
       </c>
-      <c r="D10" s="38" t="inlineStr">
+      <c r="D10" s="39" t="inlineStr">
         <is>
           <t>Config Line</t>
         </is>
       </c>
-      <c r="E10" s="38" t="inlineStr">
+      <c r="E10" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F10" s="38" t="inlineStr">
+      <c r="F10" s="39" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
@@ -4127,7 +4585,7 @@
           <t>commands: showpasswordpolicy, showsnmp, showsyslog, showaudit, showtime</t>
         </is>
       </c>
-      <c r="D11" s="40" t="inlineStr"/>
+      <c r="D11" s="41" t="inlineStr"/>
       <c r="E11" s="21" t="inlineStr">
         <is>
           <t>The following security baseline commands returned 'invalid command name' on this firmware version: showpasswordpolicy, showsnmp, showsyslog, showaudit, showtime. Password policy, SNMP configuration, syslog/audit logging, and time synchronization cannot be verified from the CLI, leaving key security controls in an unknown compliance state.</t>
@@ -4155,7 +4613,7 @@
           <t>[Banner] section empty</t>
         </is>
       </c>
-      <c r="D12" s="39" t="inlineStr">
+      <c r="D12" s="40" t="inlineStr">
         <is>
           <t>377</t>
         </is>
@@ -4187,7 +4645,7 @@
           <t>[Banner] section empty</t>
         </is>
       </c>
-      <c r="D13" s="40" t="inlineStr">
+      <c r="D13" s="41" t="inlineStr">
         <is>
           <t>375</t>
         </is>
@@ -4204,39 +4662,39 @@
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="37" t="inlineStr">
+      <c r="A15" s="38" t="inlineStr">
         <is>
           <t>CIS 4.8 — Disable Unnecessary Services on Enterprise Assets and Software</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="38" t="inlineStr">
+      <c r="A16" s="39" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B16" s="38" t="inlineStr">
+      <c r="B16" s="39" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C16" s="38" t="inlineStr">
+      <c r="C16" s="39" t="inlineStr">
         <is>
           <t>Object / Interface</t>
         </is>
       </c>
-      <c r="D16" s="38" t="inlineStr">
+      <c r="D16" s="39" t="inlineStr">
         <is>
           <t>Config Line</t>
         </is>
       </c>
-      <c r="E16" s="38" t="inlineStr">
+      <c r="E16" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F16" s="38" t="inlineStr">
+      <c r="F16" s="39" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
@@ -4258,7 +4716,7 @@
           <t>WSAPI: Enabled / Active on HTTPS 443</t>
         </is>
       </c>
-      <c r="D17" s="40" t="inlineStr"/>
+      <c r="D17" s="41" t="inlineStr"/>
       <c r="E17" s="21" t="inlineStr">
         <is>
           <t>The HP Alletra MP REST API (WSAPI) is enabled and active on HTTPS 443. The REST API exposes full array management including volume creation, deletion, VLUN mapping, and host definitions. Unauthorized access allows complete storage compromise without FC fabric access.</t>
@@ -4271,53 +4729,53 @@
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="37" t="inlineStr">
+      <c r="A19" s="38" t="inlineStr">
         <is>
           <t>CIS 5.2 — Use Unique Passwords</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="41" t="inlineStr">
+      <c r="A20" s="42" t="inlineStr">
         <is>
           <t>No findings for this control</t>
         </is>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="37" t="inlineStr">
+      <c r="A22" s="38" t="inlineStr">
         <is>
           <t>CIS 8.2 — Collect Audit Logs</t>
         </is>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="38" t="inlineStr">
+      <c r="A23" s="39" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B23" s="38" t="inlineStr">
+      <c r="B23" s="39" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C23" s="38" t="inlineStr">
+      <c r="C23" s="39" t="inlineStr">
         <is>
           <t>Object / Interface</t>
         </is>
       </c>
-      <c r="D23" s="38" t="inlineStr">
+      <c r="D23" s="39" t="inlineStr">
         <is>
           <t>Config Line</t>
         </is>
       </c>
-      <c r="E23" s="38" t="inlineStr">
+      <c r="E23" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F23" s="38" t="inlineStr">
+      <c r="F23" s="39" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
@@ -4339,7 +4797,7 @@
           <t>commands: showpasswordpolicy, showsnmp, showsyslog, showaudit, showtime</t>
         </is>
       </c>
-      <c r="D24" s="39" t="inlineStr"/>
+      <c r="D24" s="40" t="inlineStr"/>
       <c r="E24" s="20" t="inlineStr">
         <is>
           <t>The following security baseline commands returned 'invalid command name' on this firmware version: showpasswordpolicy, showsnmp, showsyslog, showaudit, showtime. Password policy, SNMP configuration, syslog/audit logging, and time synchronization cannot be verified from the CLI, leaving key security controls in an unknown compliance state.</t>
@@ -4367,7 +4825,7 @@
           <t>maps.activePolicy: dflt_base_policy</t>
         </is>
       </c>
-      <c r="D25" s="40" t="inlineStr"/>
+      <c r="D25" s="41" t="inlineStr"/>
       <c r="E25" s="21" t="inlineStr">
         <is>
           <t>MAPS is using the default policy 'dflt_base_policy' rather than a customized environment-specific policy. Default thresholds may not match this fabric's traffic patterns, causing missed alerts or excessive noise.</t>
@@ -4395,7 +4853,7 @@
           <t>maps.activePolicy: dflt_base_policy</t>
         </is>
       </c>
-      <c r="D26" s="39" t="inlineStr"/>
+      <c r="D26" s="40" t="inlineStr"/>
       <c r="E26" s="20" t="inlineStr">
         <is>
           <t>MAPS is using the default policy 'dflt_base_policy' rather than a customized environment-specific policy. Default thresholds may not match this fabric's traffic patterns, causing missed alerts or excessive noise.</t>
@@ -4408,53 +4866,53 @@
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="37" t="inlineStr">
+      <c r="A28" s="38" t="inlineStr">
         <is>
           <t>CIS 8.9 — Centralize Audit Logs</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="41" t="inlineStr">
+      <c r="A29" s="42" t="inlineStr">
         <is>
           <t>No findings for this control</t>
         </is>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="37" t="inlineStr">
+      <c r="A31" s="38" t="inlineStr">
         <is>
           <t>CIS 11.1 — Establish and Maintain a Data Recovery Practice</t>
         </is>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="38" t="inlineStr">
+      <c r="A32" s="39" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B32" s="38" t="inlineStr">
+      <c r="B32" s="39" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C32" s="38" t="inlineStr">
+      <c r="C32" s="39" t="inlineStr">
         <is>
           <t>Object / Interface</t>
         </is>
       </c>
-      <c r="D32" s="38" t="inlineStr">
+      <c r="D32" s="39" t="inlineStr">
         <is>
           <t>Config Line</t>
         </is>
       </c>
-      <c r="E32" s="38" t="inlineStr">
+      <c r="E32" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F32" s="38" t="inlineStr">
+      <c r="F32" s="39" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
@@ -4476,7 +4934,7 @@
           <t>Volume Set: DevTest1</t>
         </is>
       </c>
-      <c r="D33" s="40" t="inlineStr"/>
+      <c r="D33" s="41" t="inlineStr"/>
       <c r="E33" s="21" t="inlineStr">
         <is>
           <t>Volume set 'DevTest1' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
@@ -4504,7 +4962,7 @@
           <t>Volume Set: Infrastructure1</t>
         </is>
       </c>
-      <c r="D34" s="39" t="inlineStr"/>
+      <c r="D34" s="40" t="inlineStr"/>
       <c r="E34" s="20" t="inlineStr">
         <is>
           <t>Volume set 'Infrastructure1' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
@@ -4532,7 +4990,7 @@
           <t>Volume Set: Infrastructure2</t>
         </is>
       </c>
-      <c r="D35" s="40" t="inlineStr"/>
+      <c r="D35" s="41" t="inlineStr"/>
       <c r="E35" s="21" t="inlineStr">
         <is>
           <t>Volume set 'Infrastructure2' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
@@ -4560,7 +5018,7 @@
           <t>Volume Set: Production1</t>
         </is>
       </c>
-      <c r="D36" s="39" t="inlineStr"/>
+      <c r="D36" s="40" t="inlineStr"/>
       <c r="E36" s="20" t="inlineStr">
         <is>
           <t>Volume set 'Production1' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
@@ -4588,7 +5046,7 @@
           <t>Volume Set: Production2</t>
         </is>
       </c>
-      <c r="D37" s="40" t="inlineStr"/>
+      <c r="D37" s="41" t="inlineStr"/>
       <c r="E37" s="21" t="inlineStr">
         <is>
           <t>Volume set 'Production2' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
@@ -4601,39 +5059,39 @@
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="37" t="inlineStr">
+      <c r="A39" s="38" t="inlineStr">
         <is>
           <t>CIS 11.2 — Perform Automated Backups</t>
         </is>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="38" t="inlineStr">
+      <c r="A40" s="39" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B40" s="38" t="inlineStr">
+      <c r="B40" s="39" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C40" s="38" t="inlineStr">
+      <c r="C40" s="39" t="inlineStr">
         <is>
           <t>Object / Interface</t>
         </is>
       </c>
-      <c r="D40" s="38" t="inlineStr">
+      <c r="D40" s="39" t="inlineStr">
         <is>
           <t>Config Line</t>
         </is>
       </c>
-      <c r="E40" s="38" t="inlineStr">
+      <c r="E40" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F40" s="38" t="inlineStr">
+      <c r="F40" s="39" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
@@ -4655,7 +5113,7 @@
           <t>Volume Set: DevTest1</t>
         </is>
       </c>
-      <c r="D41" s="40" t="inlineStr"/>
+      <c r="D41" s="41" t="inlineStr"/>
       <c r="E41" s="21" t="inlineStr">
         <is>
           <t>Volume set 'DevTest1' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
@@ -4683,7 +5141,7 @@
           <t>Volume Set: Infrastructure1</t>
         </is>
       </c>
-      <c r="D42" s="39" t="inlineStr"/>
+      <c r="D42" s="40" t="inlineStr"/>
       <c r="E42" s="20" t="inlineStr">
         <is>
           <t>Volume set 'Infrastructure1' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
@@ -4711,7 +5169,7 @@
           <t>Volume Set: Infrastructure2</t>
         </is>
       </c>
-      <c r="D43" s="40" t="inlineStr"/>
+      <c r="D43" s="41" t="inlineStr"/>
       <c r="E43" s="21" t="inlineStr">
         <is>
           <t>Volume set 'Infrastructure2' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
@@ -4739,7 +5197,7 @@
           <t>Volume Set: Production1</t>
         </is>
       </c>
-      <c r="D44" s="39" t="inlineStr"/>
+      <c r="D44" s="40" t="inlineStr"/>
       <c r="E44" s="20" t="inlineStr">
         <is>
           <t>Volume set 'Production1' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
@@ -4767,7 +5225,7 @@
           <t>Volume Set: Production2</t>
         </is>
       </c>
-      <c r="D45" s="40" t="inlineStr"/>
+      <c r="D45" s="41" t="inlineStr"/>
       <c r="E45" s="21" t="inlineStr">
         <is>
           <t>Volume set 'Production2' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
@@ -4780,39 +5238,39 @@
       </c>
     </row>
     <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="37" t="inlineStr">
+      <c r="A47" s="38" t="inlineStr">
         <is>
           <t>CIS 12.2 — Establish and Maintain a Secure Network Architecture</t>
         </is>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="38" t="inlineStr">
+      <c r="A48" s="39" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B48" s="38" t="inlineStr">
+      <c r="B48" s="39" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C48" s="38" t="inlineStr">
+      <c r="C48" s="39" t="inlineStr">
         <is>
           <t>Object / Interface</t>
         </is>
       </c>
-      <c r="D48" s="38" t="inlineStr">
+      <c r="D48" s="39" t="inlineStr">
         <is>
           <t>Config Line</t>
         </is>
       </c>
-      <c r="E48" s="38" t="inlineStr">
+      <c r="E48" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F48" s="38" t="inlineStr">
+      <c r="F48" s="39" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
@@ -4834,7 +5292,7 @@
           <t>auth.policy: 0 (off)</t>
         </is>
       </c>
-      <c r="D49" s="40" t="inlineStr">
+      <c r="D49" s="41" t="inlineStr">
         <is>
           <t>22</t>
         </is>
@@ -4866,7 +5324,7 @@
           <t>defzone: allaccess</t>
         </is>
       </c>
-      <c r="D50" s="39" t="inlineStr">
+      <c r="D50" s="40" t="inlineStr">
         <is>
           <t>359</t>
         </is>
@@ -4898,7 +5356,7 @@
           <t>auth.policy: 0 (off)</t>
         </is>
       </c>
-      <c r="D51" s="40" t="inlineStr">
+      <c r="D51" s="41" t="inlineStr">
         <is>
           <t>22</t>
         </is>
@@ -4930,7 +5388,7 @@
           <t>defzone: allaccess</t>
         </is>
       </c>
-      <c r="D52" s="39" t="inlineStr">
+      <c r="D52" s="40" t="inlineStr">
         <is>
           <t>357</t>
         </is>
@@ -4962,7 +5420,7 @@
           <t>5 host(s) without CHAP</t>
         </is>
       </c>
-      <c r="D53" s="40" t="inlineStr"/>
+      <c r="D53" s="41" t="inlineStr"/>
       <c r="E53" s="21" t="inlineStr">
         <is>
           <t>No CHAP authentication is configured for 5 ESX host(s): ESX02, ESX04, ESX05, ESX06, ESX07. Both Initiator CHAP and Target CHAP show '--' in 'showhost -chap'. Without CHAP, any host presenting the correct WWN can authenticate to the array. In a compromised or miscabled environment this allows unauthorized LUN access.</t>
@@ -4990,7 +5448,7 @@
           <t>4 orphaned zone(s)</t>
         </is>
       </c>
-      <c r="D54" s="39" t="inlineStr">
+      <c r="D54" s="40" t="inlineStr">
         <is>
           <t>419</t>
         </is>
@@ -5022,7 +5480,7 @@
           <t>5 orphaned zone(s)</t>
         </is>
       </c>
-      <c r="D55" s="40" t="inlineStr">
+      <c r="D55" s="41" t="inlineStr">
         <is>
           <t>417</t>
         </is>
@@ -5054,7 +5512,7 @@
           <t>loss_sync: 0:3:2, 0:3:4, 1:3:2, 1:3:4</t>
         </is>
       </c>
-      <c r="D56" s="39" t="inlineStr"/>
+      <c r="D56" s="40" t="inlineStr"/>
       <c r="E56" s="20" t="inlineStr">
         <is>
           <t>4 FC port(s) are in 'loss_sync' state: 0:3:2, 0:3:4, 1:3:2, 1:3:4. These ports have lost synchronization with their SAN fabric counterpart and are not passing traffic. This reduces path redundancy and may indicate a cabling, SFP, or switch-side fault.</t>
@@ -5082,7 +5540,7 @@
           <t>5 FC disk(s)</t>
         </is>
       </c>
-      <c r="D57" s="40" t="inlineStr"/>
+      <c r="D57" s="41" t="inlineStr"/>
       <c r="E57" s="21" t="inlineStr">
         <is>
           <t>5 FC storage device(s) have 'Perennially Reserved' = 'No'. For FC LUNs not consumed as VMFS datastores on this host, this causes unnecessary SCSI reservation probes and path thrashing at host boot.</t>
@@ -5095,39 +5553,39 @@
       </c>
     </row>
     <row r="59" ht="22" customHeight="1">
-      <c r="A59" s="37" t="inlineStr">
+      <c r="A59" s="38" t="inlineStr">
         <is>
           <t>CIS 12.3 — Securely Manage Network Infrastructure</t>
         </is>
       </c>
     </row>
     <row r="60" ht="20" customHeight="1">
-      <c r="A60" s="38" t="inlineStr">
+      <c r="A60" s="39" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B60" s="38" t="inlineStr">
+      <c r="B60" s="39" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C60" s="38" t="inlineStr">
+      <c r="C60" s="39" t="inlineStr">
         <is>
           <t>Object / Interface</t>
         </is>
       </c>
-      <c r="D60" s="38" t="inlineStr">
+      <c r="D60" s="39" t="inlineStr">
         <is>
           <t>Config Line</t>
         </is>
       </c>
-      <c r="E60" s="38" t="inlineStr">
+      <c r="E60" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F60" s="38" t="inlineStr">
+      <c r="F60" s="39" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
@@ -5149,7 +5607,7 @@
           <t>auth.policy: 0 (off)</t>
         </is>
       </c>
-      <c r="D61" s="40" t="inlineStr">
+      <c r="D61" s="41" t="inlineStr">
         <is>
           <t>22</t>
         </is>
@@ -5181,7 +5639,7 @@
           <t>auth.policy: 0 (off)</t>
         </is>
       </c>
-      <c r="D62" s="39" t="inlineStr">
+      <c r="D62" s="40" t="inlineStr">
         <is>
           <t>22</t>
         </is>
@@ -5213,7 +5671,7 @@
           <t>WSAPI: Enabled / Active on HTTPS 443</t>
         </is>
       </c>
-      <c r="D63" s="40" t="inlineStr"/>
+      <c r="D63" s="41" t="inlineStr"/>
       <c r="E63" s="21" t="inlineStr">
         <is>
           <t>The HP Alletra MP REST API (WSAPI) is enabled and active on HTTPS 443. The REST API exposes full array management including volume creation, deletion, VLUN mapping, and host definitions. Unauthorized access allows complete storage compromise without FC fabric access.</t>
@@ -5226,39 +5684,39 @@
       </c>
     </row>
     <row r="65" ht="22" customHeight="1">
-      <c r="A65" s="37" t="inlineStr">
+      <c r="A65" s="38" t="inlineStr">
         <is>
           <t>CIS 12.6 — Use Secure Network Management and Communication Protocols</t>
         </is>
       </c>
     </row>
     <row r="66" ht="20" customHeight="1">
-      <c r="A66" s="38" t="inlineStr">
+      <c r="A66" s="39" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B66" s="38" t="inlineStr">
+      <c r="B66" s="39" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C66" s="38" t="inlineStr">
+      <c r="C66" s="39" t="inlineStr">
         <is>
           <t>Object / Interface</t>
         </is>
       </c>
-      <c r="D66" s="38" t="inlineStr">
+      <c r="D66" s="39" t="inlineStr">
         <is>
           <t>Config Line</t>
         </is>
       </c>
-      <c r="E66" s="38" t="inlineStr">
+      <c r="E66" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F66" s="38" t="inlineStr">
+      <c r="F66" s="39" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
@@ -5280,7 +5738,7 @@
           <t>showsshkey: No SSH key found</t>
         </is>
       </c>
-      <c r="D67" s="40" t="inlineStr"/>
+      <c r="D67" s="41" t="inlineStr"/>
       <c r="E67" s="21" t="inlineStr">
         <is>
           <t>No SSH public keys are configured on the Alletra MP. Administrative access relies exclusively on password authentication. Password-only authentication is weaker than key-based auth and does not meet PCI DSS requirements for strong cryptographic access controls.</t>
@@ -5293,39 +5751,39 @@
       </c>
     </row>
     <row r="69" ht="22" customHeight="1">
-      <c r="A69" s="37" t="inlineStr">
+      <c r="A69" s="38" t="inlineStr">
         <is>
           <t>CIS 13.4 — Perform Traffic Filtering Between Network Segments</t>
         </is>
       </c>
     </row>
     <row r="70" ht="20" customHeight="1">
-      <c r="A70" s="38" t="inlineStr">
+      <c r="A70" s="39" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B70" s="38" t="inlineStr">
+      <c r="B70" s="39" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C70" s="38" t="inlineStr">
+      <c r="C70" s="39" t="inlineStr">
         <is>
           <t>Object / Interface</t>
         </is>
       </c>
-      <c r="D70" s="38" t="inlineStr">
+      <c r="D70" s="39" t="inlineStr">
         <is>
           <t>Config Line</t>
         </is>
       </c>
-      <c r="E70" s="38" t="inlineStr">
+      <c r="E70" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F70" s="38" t="inlineStr">
+      <c r="F70" s="39" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
@@ -5347,7 +5805,7 @@
           <t>defzone: allaccess</t>
         </is>
       </c>
-      <c r="D71" s="40" t="inlineStr">
+      <c r="D71" s="41" t="inlineStr">
         <is>
           <t>359</t>
         </is>
@@ -5379,7 +5837,7 @@
           <t>defzone: allaccess</t>
         </is>
       </c>
-      <c r="D72" s="39" t="inlineStr">
+      <c r="D72" s="40" t="inlineStr">
         <is>
           <t>357</t>
         </is>
@@ -5436,7 +5894,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="42" t="inlineStr">
+      <c r="A1" s="43" t="inlineStr">
         <is>
           <t>PCI DSS v4.0 — Finding Cross-Reference</t>
         </is>
@@ -5450,39 +5908,39 @@
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="43" t="inlineStr">
+      <c r="A3" s="44" t="inlineStr">
         <is>
           <t>PCI DSS 1.2.4  [5 findings]  All traffic between trusted/untrusted networks is explicitly controlled</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="38" t="inlineStr">
+      <c r="A4" s="39" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B4" s="38" t="inlineStr">
+      <c r="B4" s="39" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C4" s="38" t="inlineStr">
+      <c r="C4" s="39" t="inlineStr">
         <is>
           <t>Object / Interface</t>
         </is>
       </c>
-      <c r="D4" s="38" t="inlineStr">
+      <c r="D4" s="39" t="inlineStr">
         <is>
           <t>Config Line</t>
         </is>
       </c>
-      <c r="E4" s="38" t="inlineStr">
+      <c r="E4" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F4" s="38" t="inlineStr">
+      <c r="F4" s="39" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
@@ -5504,7 +5962,7 @@
           <t>auth.policy: 0 (off)</t>
         </is>
       </c>
-      <c r="D5" s="40" t="inlineStr">
+      <c r="D5" s="41" t="inlineStr">
         <is>
           <t>22</t>
         </is>
@@ -5536,7 +5994,7 @@
           <t>defzone: allaccess</t>
         </is>
       </c>
-      <c r="D6" s="39" t="inlineStr">
+      <c r="D6" s="40" t="inlineStr">
         <is>
           <t>359</t>
         </is>
@@ -5568,7 +6026,7 @@
           <t>auth.policy: 0 (off)</t>
         </is>
       </c>
-      <c r="D7" s="40" t="inlineStr">
+      <c r="D7" s="41" t="inlineStr">
         <is>
           <t>22</t>
         </is>
@@ -5600,7 +6058,7 @@
           <t>defzone: allaccess</t>
         </is>
       </c>
-      <c r="D8" s="39" t="inlineStr">
+      <c r="D8" s="40" t="inlineStr">
         <is>
           <t>357</t>
         </is>
@@ -5632,7 +6090,7 @@
           <t>5 host(s) without CHAP</t>
         </is>
       </c>
-      <c r="D9" s="40" t="inlineStr"/>
+      <c r="D9" s="41" t="inlineStr"/>
       <c r="E9" s="21" t="inlineStr">
         <is>
           <t>No CHAP authentication is configured for 5 ESX host(s): ESX02, ESX04, ESX05, ESX06, ESX07. Both Initiator CHAP and Target CHAP show '--' in 'showhost -chap'. Without CHAP, any host presenting the correct WWN can authenticate to the array. In a compromised or miscabled environment this allows unauthorized LUN access.</t>
@@ -5645,39 +6103,39 @@
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="43" t="inlineStr">
+      <c r="A11" s="44" t="inlineStr">
         <is>
           <t>PCI DSS 1.3.2  [2 findings]  Outbound traffic from the CDE is restricted to only that which is necessary</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="38" t="inlineStr">
+      <c r="A12" s="39" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B12" s="38" t="inlineStr">
+      <c r="B12" s="39" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C12" s="38" t="inlineStr">
+      <c r="C12" s="39" t="inlineStr">
         <is>
           <t>Object / Interface</t>
         </is>
       </c>
-      <c r="D12" s="38" t="inlineStr">
+      <c r="D12" s="39" t="inlineStr">
         <is>
           <t>Config Line</t>
         </is>
       </c>
-      <c r="E12" s="38" t="inlineStr">
+      <c r="E12" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F12" s="38" t="inlineStr">
+      <c r="F12" s="39" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
@@ -5699,7 +6157,7 @@
           <t>defzone: allaccess</t>
         </is>
       </c>
-      <c r="D13" s="40" t="inlineStr">
+      <c r="D13" s="41" t="inlineStr">
         <is>
           <t>359</t>
         </is>
@@ -5731,7 +6189,7 @@
           <t>defzone: allaccess</t>
         </is>
       </c>
-      <c r="D14" s="39" t="inlineStr">
+      <c r="D14" s="40" t="inlineStr">
         <is>
           <t>357</t>
         </is>
@@ -5748,39 +6206,39 @@
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="43" t="inlineStr">
+      <c r="A16" s="44" t="inlineStr">
         <is>
           <t>PCI DSS 2.2.1  [3 findings]  Configuration standards are defined for all system components</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="38" t="inlineStr">
+      <c r="A17" s="39" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B17" s="38" t="inlineStr">
+      <c r="B17" s="39" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C17" s="38" t="inlineStr">
+      <c r="C17" s="39" t="inlineStr">
         <is>
           <t>Object / Interface</t>
         </is>
       </c>
-      <c r="D17" s="38" t="inlineStr">
+      <c r="D17" s="39" t="inlineStr">
         <is>
           <t>Config Line</t>
         </is>
       </c>
-      <c r="E17" s="38" t="inlineStr">
+      <c r="E17" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F17" s="38" t="inlineStr">
+      <c r="F17" s="39" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
@@ -5802,7 +6260,7 @@
           <t>commands: showpasswordpolicy, showsnmp, showsyslog, showaudit, showtime</t>
         </is>
       </c>
-      <c r="D18" s="39" t="inlineStr"/>
+      <c r="D18" s="40" t="inlineStr"/>
       <c r="E18" s="20" t="inlineStr">
         <is>
           <t>The following security baseline commands returned 'invalid command name' on this firmware version: showpasswordpolicy, showsnmp, showsyslog, showaudit, showtime. Password policy, SNMP configuration, syslog/audit logging, and time synchronization cannot be verified from the CLI, leaving key security controls in an unknown compliance state.</t>
@@ -5830,7 +6288,7 @@
           <t>[Banner] section empty</t>
         </is>
       </c>
-      <c r="D19" s="40" t="inlineStr">
+      <c r="D19" s="41" t="inlineStr">
         <is>
           <t>377</t>
         </is>
@@ -5862,7 +6320,7 @@
           <t>[Banner] section empty</t>
         </is>
       </c>
-      <c r="D20" s="39" t="inlineStr">
+      <c r="D20" s="40" t="inlineStr">
         <is>
           <t>375</t>
         </is>
@@ -5879,39 +6337,39 @@
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="43" t="inlineStr">
+      <c r="A22" s="44" t="inlineStr">
         <is>
           <t>PCI DSS 2.2.4  [1 finding]  Only necessary services, protocols, and functions are enabled</t>
         </is>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="38" t="inlineStr">
+      <c r="A23" s="39" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B23" s="38" t="inlineStr">
+      <c r="B23" s="39" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C23" s="38" t="inlineStr">
+      <c r="C23" s="39" t="inlineStr">
         <is>
           <t>Object / Interface</t>
         </is>
       </c>
-      <c r="D23" s="38" t="inlineStr">
+      <c r="D23" s="39" t="inlineStr">
         <is>
           <t>Config Line</t>
         </is>
       </c>
-      <c r="E23" s="38" t="inlineStr">
+      <c r="E23" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F23" s="38" t="inlineStr">
+      <c r="F23" s="39" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
@@ -5933,7 +6391,7 @@
           <t>WSAPI: Enabled / Active on HTTPS 443</t>
         </is>
       </c>
-      <c r="D24" s="39" t="inlineStr"/>
+      <c r="D24" s="40" t="inlineStr"/>
       <c r="E24" s="20" t="inlineStr">
         <is>
           <t>The HP Alletra MP REST API (WSAPI) is enabled and active on HTTPS 443. The REST API exposes full array management including volume creation, deletion, VLUN mapping, and host definitions. Unauthorized access allows complete storage compromise without FC fabric access.</t>
@@ -5946,39 +6404,39 @@
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="43" t="inlineStr">
+      <c r="A26" s="44" t="inlineStr">
         <is>
           <t>PCI DSS 2.2.7  [1 finding]  All non-console administrative access is encrypted using strong cryptography</t>
         </is>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="38" t="inlineStr">
+      <c r="A27" s="39" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B27" s="38" t="inlineStr">
+      <c r="B27" s="39" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C27" s="38" t="inlineStr">
+      <c r="C27" s="39" t="inlineStr">
         <is>
           <t>Object / Interface</t>
         </is>
       </c>
-      <c r="D27" s="38" t="inlineStr">
+      <c r="D27" s="39" t="inlineStr">
         <is>
           <t>Config Line</t>
         </is>
       </c>
-      <c r="E27" s="38" t="inlineStr">
+      <c r="E27" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F27" s="38" t="inlineStr">
+      <c r="F27" s="39" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
@@ -6000,7 +6458,7 @@
           <t>showsshkey: No SSH key found</t>
         </is>
       </c>
-      <c r="D28" s="39" t="inlineStr"/>
+      <c r="D28" s="40" t="inlineStr"/>
       <c r="E28" s="20" t="inlineStr">
         <is>
           <t>No SSH public keys are configured on the Alletra MP. Administrative access relies exclusively on password authentication. Password-only authentication is weaker than key-based auth and does not meet PCI DSS requirements for strong cryptographic access controls.</t>
@@ -6013,39 +6471,39 @@
       </c>
     </row>
     <row r="30" ht="28" customHeight="1">
-      <c r="A30" s="43" t="inlineStr">
+      <c r="A30" s="44" t="inlineStr">
         <is>
           <t>PCI DSS 4.2.1  [4 findings]  Strong cryptography safeguards transmission of cardholder data</t>
         </is>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="38" t="inlineStr">
+      <c r="A31" s="39" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B31" s="38" t="inlineStr">
+      <c r="B31" s="39" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C31" s="38" t="inlineStr">
+      <c r="C31" s="39" t="inlineStr">
         <is>
           <t>Object / Interface</t>
         </is>
       </c>
-      <c r="D31" s="38" t="inlineStr">
+      <c r="D31" s="39" t="inlineStr">
         <is>
           <t>Config Line</t>
         </is>
       </c>
-      <c r="E31" s="38" t="inlineStr">
+      <c r="E31" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F31" s="38" t="inlineStr">
+      <c r="F31" s="39" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
@@ -6067,7 +6525,7 @@
           <t>auth.policy: 0 (off)</t>
         </is>
       </c>
-      <c r="D32" s="39" t="inlineStr">
+      <c r="D32" s="40" t="inlineStr">
         <is>
           <t>22</t>
         </is>
@@ -6099,7 +6557,7 @@
           <t>auth.policy: 0 (off)</t>
         </is>
       </c>
-      <c r="D33" s="40" t="inlineStr">
+      <c r="D33" s="41" t="inlineStr">
         <is>
           <t>22</t>
         </is>
@@ -6131,7 +6589,7 @@
           <t>5 host(s) without CHAP</t>
         </is>
       </c>
-      <c r="D34" s="39" t="inlineStr"/>
+      <c r="D34" s="40" t="inlineStr"/>
       <c r="E34" s="20" t="inlineStr">
         <is>
           <t>No CHAP authentication is configured for 5 ESX host(s): ESX02, ESX04, ESX05, ESX06, ESX07. Both Initiator CHAP and Target CHAP show '--' in 'showhost -chap'. Without CHAP, any host presenting the correct WWN can authenticate to the array. In a compromised or miscabled environment this allows unauthorized LUN access.</t>
@@ -6159,7 +6617,7 @@
           <t>showsshkey: No SSH key found</t>
         </is>
       </c>
-      <c r="D35" s="40" t="inlineStr"/>
+      <c r="D35" s="41" t="inlineStr"/>
       <c r="E35" s="21" t="inlineStr">
         <is>
           <t>No SSH public keys are configured on the Alletra MP. Administrative access relies exclusively on password authentication. Password-only authentication is weaker than key-based auth and does not meet PCI DSS requirements for strong cryptographic access controls.</t>
@@ -6172,39 +6630,39 @@
       </c>
     </row>
     <row r="37" ht="28" customHeight="1">
-      <c r="A37" s="43" t="inlineStr">
+      <c r="A37" s="44" t="inlineStr">
         <is>
           <t>PCI DSS 10.5.4  [1 finding]  Audit log files are protected to prevent unauthorized access or modifications</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="38" t="inlineStr">
+      <c r="A38" s="39" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B38" s="38" t="inlineStr">
+      <c r="B38" s="39" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C38" s="38" t="inlineStr">
+      <c r="C38" s="39" t="inlineStr">
         <is>
           <t>Object / Interface</t>
         </is>
       </c>
-      <c r="D38" s="38" t="inlineStr">
+      <c r="D38" s="39" t="inlineStr">
         <is>
           <t>Config Line</t>
         </is>
       </c>
-      <c r="E38" s="38" t="inlineStr">
+      <c r="E38" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F38" s="38" t="inlineStr">
+      <c r="F38" s="39" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
@@ -6226,7 +6684,7 @@
           <t>commands: showpasswordpolicy, showsnmp, showsyslog, showaudit, showtime</t>
         </is>
       </c>
-      <c r="D39" s="40" t="inlineStr"/>
+      <c r="D39" s="41" t="inlineStr"/>
       <c r="E39" s="21" t="inlineStr">
         <is>
           <t>The following security baseline commands returned 'invalid command name' on this firmware version: showpasswordpolicy, showsnmp, showsyslog, showaudit, showtime. Password policy, SNMP configuration, syslog/audit logging, and time synchronization cannot be verified from the CLI, leaving key security controls in an unknown compliance state.</t>

</xml_diff>

<commit_message>
Add source_file to Asset column for 'filename: devicename' format
All parser run_checks() methods now pass source_file=os.path.basename(self.path)
to IssueStore.add(). The Security Issues Asset column now shows
"<filename>: <devicename>" to make the evidence source immediately clear.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/san/sample-san_analysis.xlsx
+++ b/san/sample-san_analysis.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCI DSS Mapping" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Security Issues'!$A$1:$N$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Security Issues'!$A$1:$O$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -762,7 +762,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-15 22:52:00    Switches: swd77 Domain 1; swd77 Domain 2    Array: ZZZZZ01p-mp HPE Alletra Storage</t>
+          <t>Generated: 2026-06-15 23:08:36    Switches: swd77 Domain 1; swd77 Domain 2    Array: ZZZZZ01p-mp HPE Alletra Storage</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2954,10 +2954,11 @@
     <col width="60" customWidth="1" min="8" max="8"/>
     <col width="60" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="36" customWidth="1" min="13" max="13"/>
-    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="36" customWidth="1" min="14" max="14"/>
+    <col width="34" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -3013,20 +3014,25 @@
       </c>
       <c r="K1" s="9" t="inlineStr">
         <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="L1" s="9" t="inlineStr">
+        <is>
           <t>Verified</t>
         </is>
       </c>
-      <c r="L1" s="9" t="inlineStr">
+      <c r="M1" s="9" t="inlineStr">
         <is>
           <t>Asset</t>
         </is>
       </c>
-      <c r="M1" s="9" t="inlineStr">
+      <c r="N1" s="9" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="N1" s="9" t="inlineStr">
+      <c r="O1" s="9" t="inlineStr">
         <is>
           <t>Vuln</t>
         </is>
@@ -3068,7 +3074,7 @@
       </c>
       <c r="H2" s="20" t="inlineStr">
         <is>
-          <t>FC Authentication Policy is disabled (auth.policy=0). No DH-CHAP authentication is required between fabric ports. An unauthorized switch or rogue HBA can join the fabric without credentials, enabling eavesdropping and spoofed SCSI commands on VMware datastores.</t>
+          <t>FC Authentication Policy (DH-CHAP) is disabled. No authentication is required between fabric ports, allowing unauthorized switches or rogue HBAs to join the fabric without credentials and enabling fabric eavesdropping and spoofed SCSI commands.</t>
         </is>
       </c>
       <c r="I2" s="20" t="inlineStr">
@@ -3081,22 +3087,27 @@
           <t>configShow line 22</t>
         </is>
       </c>
-      <c r="K2" s="33" t="inlineStr">
+      <c r="K2" s="20" t="inlineStr">
+        <is>
+          <t>configShow: auth.policy=0 (off) at line 22. DH-CHAP authentication is not enforced on any fabric port. Active config: ZZZZZG_SAN_A.</t>
+        </is>
+      </c>
+      <c r="L2" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L2" s="20" t="inlineStr">
-        <is>
-          <t>swd77 (Domain 1)</t>
-        </is>
-      </c>
       <c r="M2" s="20" t="inlineStr">
         <is>
+          <t>Brocade01 2026-06-01.log: swd77 (Domain 1)</t>
+        </is>
+      </c>
+      <c r="N2" s="20" t="inlineStr">
+        <is>
           <t>auth.policy: 0 (off) (22)</t>
         </is>
       </c>
-      <c r="N2" s="20" t="inlineStr">
+      <c r="O2" s="20" t="inlineStr">
         <is>
           <t>SAN - FC Authentication Policy Disabled</t>
         </is>
@@ -3138,7 +3149,7 @@
       </c>
       <c r="H3" s="21" t="inlineStr">
         <is>
-          <t>The default zone is set to 'allaccess'. Any device not placed in a named zone can communicate with ALL other unzoned devices, creating an open fabric. A rogue HBA inserted into any open port gains full fabric visibility. This violates SAN isolation requirements for VMware.</t>
+          <t>The default zone policy is set to 'allaccess'. Devices not placed in a named zone can communicate with all other unzoned devices, creating an open fabric with no isolation between initiators and targets.</t>
         </is>
       </c>
       <c r="I3" s="21" t="inlineStr">
@@ -3151,22 +3162,27 @@
           <t>configShow line 359</t>
         </is>
       </c>
-      <c r="K3" s="33" t="inlineStr">
+      <c r="K3" s="21" t="inlineStr">
+        <is>
+          <t>configShow: defzone=allaccess at line 359. Active config: ZZZZZG_SAN_A. All fabric ports without explicit zone membership have unrestricted access.</t>
+        </is>
+      </c>
+      <c r="L3" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L3" s="21" t="inlineStr">
-        <is>
-          <t>swd77 (Domain 1)</t>
-        </is>
-      </c>
       <c r="M3" s="21" t="inlineStr">
         <is>
+          <t>Brocade01 2026-06-01.log: swd77 (Domain 1)</t>
+        </is>
+      </c>
+      <c r="N3" s="21" t="inlineStr">
+        <is>
           <t>defzone: allaccess (359)</t>
         </is>
       </c>
-      <c r="N3" s="21" t="inlineStr">
+      <c r="O3" s="21" t="inlineStr">
         <is>
           <t>SAN - Default Zone Allows All Access</t>
         </is>
@@ -3208,7 +3224,7 @@
       </c>
       <c r="H4" s="20" t="inlineStr">
         <is>
-          <t>FC Authentication Policy is disabled (auth.policy=0). No DH-CHAP authentication is required between fabric ports. An unauthorized switch or rogue HBA can join the fabric without credentials, enabling eavesdropping and spoofed SCSI commands on VMware datastores.</t>
+          <t>FC Authentication Policy (DH-CHAP) is disabled. No authentication is required between fabric ports, allowing unauthorized switches or rogue HBAs to join the fabric without credentials and enabling fabric eavesdropping and spoofed SCSI commands.</t>
         </is>
       </c>
       <c r="I4" s="20" t="inlineStr">
@@ -3221,22 +3237,27 @@
           <t>configShow line 22</t>
         </is>
       </c>
-      <c r="K4" s="33" t="inlineStr">
+      <c r="K4" s="20" t="inlineStr">
+        <is>
+          <t>configShow: auth.policy=0 (off) at line 22. DH-CHAP authentication is not enforced on any fabric port. Active config: ZZZZZG_SAN_B.</t>
+        </is>
+      </c>
+      <c r="L4" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L4" s="20" t="inlineStr">
-        <is>
-          <t>swd77 (Domain 2)</t>
-        </is>
-      </c>
       <c r="M4" s="20" t="inlineStr">
         <is>
+          <t>Brocade02 2026-06-01.log: swd77 (Domain 2)</t>
+        </is>
+      </c>
+      <c r="N4" s="20" t="inlineStr">
+        <is>
           <t>auth.policy: 0 (off) (22)</t>
         </is>
       </c>
-      <c r="N4" s="20" t="inlineStr">
+      <c r="O4" s="20" t="inlineStr">
         <is>
           <t>SAN - FC Authentication Policy Disabled</t>
         </is>
@@ -3278,7 +3299,7 @@
       </c>
       <c r="H5" s="21" t="inlineStr">
         <is>
-          <t>The default zone is set to 'allaccess'. Any device not placed in a named zone can communicate with ALL other unzoned devices, creating an open fabric. A rogue HBA inserted into any open port gains full fabric visibility. This violates SAN isolation requirements for VMware.</t>
+          <t>The default zone policy is set to 'allaccess'. Devices not placed in a named zone can communicate with all other unzoned devices, creating an open fabric with no isolation between initiators and targets.</t>
         </is>
       </c>
       <c r="I5" s="21" t="inlineStr">
@@ -3291,22 +3312,27 @@
           <t>configShow line 357</t>
         </is>
       </c>
-      <c r="K5" s="33" t="inlineStr">
+      <c r="K5" s="21" t="inlineStr">
+        <is>
+          <t>configShow: defzone=allaccess at line 357. Active config: ZZZZZG_SAN_B. All fabric ports without explicit zone membership have unrestricted access.</t>
+        </is>
+      </c>
+      <c r="L5" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L5" s="21" t="inlineStr">
-        <is>
-          <t>swd77 (Domain 2)</t>
-        </is>
-      </c>
       <c r="M5" s="21" t="inlineStr">
         <is>
+          <t>Brocade02 2026-06-01.log: swd77 (Domain 2)</t>
+        </is>
+      </c>
+      <c r="N5" s="21" t="inlineStr">
+        <is>
           <t>defzone: allaccess (357)</t>
         </is>
       </c>
-      <c r="N5" s="21" t="inlineStr">
+      <c r="O5" s="21" t="inlineStr">
         <is>
           <t>SAN - Default Zone Allows All Access</t>
         </is>
@@ -3344,7 +3370,7 @@
       </c>
       <c r="H6" s="20" t="inlineStr">
         <is>
-          <t>No CHAP authentication is configured for 5 ESX host(s): ESX02, ESX04, ESX05, ESX06, ESX07. Both Initiator CHAP and Target CHAP show '--' in 'showhost -chap'. Without CHAP, any host presenting the correct WWN can authenticate to the array. In a compromised or miscabled environment this allows unauthorized LUN access.</t>
+          <t>No CHAP (Challenge-Handshake Authentication Protocol) authentication is configured for storage hosts. Without CHAP, any host presenting the correct WWN can authenticate to the array, enabling unauthorized LUN access in a compromised or miscabled environment.</t>
         </is>
       </c>
       <c r="I6" s="20" t="inlineStr">
@@ -3357,22 +3383,27 @@
           <t>showhost -chap: ESX02, ESX04, ESX05, ESX06, ESX07</t>
         </is>
       </c>
-      <c r="K6" s="33" t="inlineStr">
+      <c r="K6" s="20" t="inlineStr">
+        <is>
+          <t>showhost -chap: 5 host(s) show '--' (not configured) for both Initiator CHAP Name and Target CHAP Name: ESX02, ESX04, ESX05, ESX06, ESX07.</t>
+        </is>
+      </c>
+      <c r="L6" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L6" s="20" t="inlineStr">
-        <is>
-          <t>ZZZZZ01p-mp</t>
-        </is>
-      </c>
       <c r="M6" s="20" t="inlineStr">
         <is>
+          <t>Alletra 2026-06-09-01.log: ZZZZZ01p-mp</t>
+        </is>
+      </c>
+      <c r="N6" s="20" t="inlineStr">
+        <is>
           <t>5 host(s) without CHAP</t>
         </is>
       </c>
-      <c r="N6" s="20" t="inlineStr">
+      <c r="O6" s="20" t="inlineStr">
         <is>
           <t>SAN - No CHAP on Storage Hosts</t>
         </is>
@@ -3410,7 +3441,7 @@
       </c>
       <c r="H7" s="21" t="inlineStr">
         <is>
-          <t>The following security baseline commands returned 'invalid command name' on this firmware version: showpasswordpolicy, showsnmp, showsyslog, showaudit, showtime. Password policy, SNMP configuration, syslog/audit logging, and time synchronization cannot be verified from the CLI, leaving key security controls in an unknown compliance state.</t>
+          <t>Security baseline commands are not available on this firmware version. Password policy, SNMP configuration, syslog, audit logging, and time synchronization settings cannot be verified from the CLI, leaving key security controls in an unknown compliance state.</t>
         </is>
       </c>
       <c r="I7" s="21" t="inlineStr">
@@ -3423,22 +3454,27 @@
           <t>Invalid on this firmware: showpasswordpolicy, showsnmp, showsyslog, showaudit, showtime</t>
         </is>
       </c>
-      <c r="K7" s="33" t="inlineStr">
+      <c r="K7" s="21" t="inlineStr">
+        <is>
+          <t>Commands returning 'invalid command name' on this firmware: showpasswordpolicy, showsnmp, showsyslog, showaudit, showtime. These settings cannot be audited via CLI.</t>
+        </is>
+      </c>
+      <c r="L7" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L7" s="21" t="inlineStr">
-        <is>
-          <t>ZZZZZ01p-mp</t>
-        </is>
-      </c>
       <c r="M7" s="21" t="inlineStr">
         <is>
+          <t>Alletra 2026-06-09-01.log: ZZZZZ01p-mp</t>
+        </is>
+      </c>
+      <c r="N7" s="21" t="inlineStr">
+        <is>
           <t>commands: showpasswordpolicy, showsnmp, showsyslog, showaudit, showtime</t>
         </is>
       </c>
-      <c r="N7" s="21" t="inlineStr">
+      <c r="O7" s="21" t="inlineStr">
         <is>
           <t>SAN - Security Baseline Not Verifiable</t>
         </is>
@@ -3476,7 +3512,7 @@
       </c>
       <c r="H8" s="20" t="inlineStr">
         <is>
-          <t>No SSH public keys are configured on the Alletra MP. Administrative access relies exclusively on password authentication. Password-only authentication is weaker than key-based auth and does not meet PCI DSS requirements for strong cryptographic access controls.</t>
+          <t>No SSH public keys are configured on the storage array. Administrative access relies exclusively on password authentication, which does not meet requirements for strong cryptographic access controls.</t>
         </is>
       </c>
       <c r="I8" s="20" t="inlineStr">
@@ -3489,22 +3525,27 @@
           <t>showsshkey: No SSH key found</t>
         </is>
       </c>
-      <c r="K8" s="33" t="inlineStr">
+      <c r="K8" s="20" t="inlineStr">
+        <is>
+          <t>showsshkey: 'No SSH key found'. All administrative authentication uses passwords only; no public-key authentication is configured.</t>
+        </is>
+      </c>
+      <c r="L8" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L8" s="20" t="inlineStr">
-        <is>
-          <t>ZZZZZ01p-mp</t>
-        </is>
-      </c>
       <c r="M8" s="20" t="inlineStr">
         <is>
+          <t>Alletra 2026-06-09-01.log: ZZZZZ01p-mp</t>
+        </is>
+      </c>
+      <c r="N8" s="20" t="inlineStr">
+        <is>
           <t>showsshkey: No SSH key found</t>
         </is>
       </c>
-      <c r="N8" s="20" t="inlineStr">
+      <c r="O8" s="20" t="inlineStr">
         <is>
           <t>SAN - No SSH Keys Configured</t>
         </is>
@@ -3538,7 +3579,7 @@
       <c r="G9" s="36" t="inlineStr"/>
       <c r="H9" s="21" t="inlineStr">
         <is>
-          <t>Volume set 'DevTest1' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
+          <t>No remote replication is configured for this exported volume set. Local snapshots alone cannot protect against site-level failure, storage hardware failure, or ransomware that corrupts all local snapshots before a recovery point is reached.</t>
         </is>
       </c>
       <c r="I9" s="21" t="inlineStr">
@@ -3551,22 +3592,27 @@
           <t>Protection: Local Snapshots | Replication: None</t>
         </is>
       </c>
-      <c r="K9" s="33" t="inlineStr">
+      <c r="K9" s="21" t="inlineStr">
+        <is>
+          <t>Volumes CSV: Volume Set 'DevTest1' — Protection Level='Local Snapshots', Replication Type='None', Export Status=Exported. No DR replication target configured.</t>
+        </is>
+      </c>
+      <c r="L9" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L9" s="21" t="inlineStr">
-        <is>
-          <t>hai01p-mp</t>
-        </is>
-      </c>
       <c r="M9" s="21" t="inlineStr">
         <is>
+          <t>Volumes_Inventory_06092026_120519.csv: hai01p-mp</t>
+        </is>
+      </c>
+      <c r="N9" s="21" t="inlineStr">
+        <is>
           <t>Volume Set: DevTest1</t>
         </is>
       </c>
-      <c r="N9" s="21" t="inlineStr">
+      <c r="O9" s="21" t="inlineStr">
         <is>
           <t>SAN - No Volume Replication Configured</t>
         </is>
@@ -3600,7 +3646,7 @@
       <c r="G10" s="32" t="inlineStr"/>
       <c r="H10" s="20" t="inlineStr">
         <is>
-          <t>Volume set 'Infrastructure1' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
+          <t>No remote replication is configured for this exported volume set. Local snapshots alone cannot protect against site-level failure, storage hardware failure, or ransomware that corrupts all local snapshots before a recovery point is reached.</t>
         </is>
       </c>
       <c r="I10" s="20" t="inlineStr">
@@ -3613,22 +3659,27 @@
           <t>Protection: Local Snapshots | Replication: None</t>
         </is>
       </c>
-      <c r="K10" s="33" t="inlineStr">
+      <c r="K10" s="20" t="inlineStr">
+        <is>
+          <t>Volumes CSV: Volume Set 'Infrastructure1' — Protection Level='Local Snapshots', Replication Type='None', Export Status=Exported. No DR replication target configured.</t>
+        </is>
+      </c>
+      <c r="L10" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L10" s="20" t="inlineStr">
-        <is>
-          <t>hai01p-mp</t>
-        </is>
-      </c>
       <c r="M10" s="20" t="inlineStr">
         <is>
+          <t>Volumes_Inventory_06092026_120519.csv: hai01p-mp</t>
+        </is>
+      </c>
+      <c r="N10" s="20" t="inlineStr">
+        <is>
           <t>Volume Set: Infrastructure1</t>
         </is>
       </c>
-      <c r="N10" s="20" t="inlineStr">
+      <c r="O10" s="20" t="inlineStr">
         <is>
           <t>SAN - No Volume Replication Configured</t>
         </is>
@@ -3662,7 +3713,7 @@
       <c r="G11" s="36" t="inlineStr"/>
       <c r="H11" s="21" t="inlineStr">
         <is>
-          <t>Volume set 'Infrastructure2' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
+          <t>No remote replication is configured for this exported volume set. Local snapshots alone cannot protect against site-level failure, storage hardware failure, or ransomware that corrupts all local snapshots before a recovery point is reached.</t>
         </is>
       </c>
       <c r="I11" s="21" t="inlineStr">
@@ -3675,22 +3726,27 @@
           <t>Protection: Local Snapshots | Replication: None</t>
         </is>
       </c>
-      <c r="K11" s="33" t="inlineStr">
+      <c r="K11" s="21" t="inlineStr">
+        <is>
+          <t>Volumes CSV: Volume Set 'Infrastructure2' — Protection Level='Local Snapshots', Replication Type='None', Export Status=Exported. No DR replication target configured.</t>
+        </is>
+      </c>
+      <c r="L11" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L11" s="21" t="inlineStr">
-        <is>
-          <t>hai01p-mp</t>
-        </is>
-      </c>
       <c r="M11" s="21" t="inlineStr">
         <is>
+          <t>Volumes_Inventory_06092026_120519.csv: hai01p-mp</t>
+        </is>
+      </c>
+      <c r="N11" s="21" t="inlineStr">
+        <is>
           <t>Volume Set: Infrastructure2</t>
         </is>
       </c>
-      <c r="N11" s="21" t="inlineStr">
+      <c r="O11" s="21" t="inlineStr">
         <is>
           <t>SAN - No Volume Replication Configured</t>
         </is>
@@ -3724,7 +3780,7 @@
       <c r="G12" s="32" t="inlineStr"/>
       <c r="H12" s="20" t="inlineStr">
         <is>
-          <t>Volume set 'Production1' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
+          <t>No remote replication is configured for this exported volume set. Local snapshots alone cannot protect against site-level failure, storage hardware failure, or ransomware that corrupts all local snapshots before a recovery point is reached.</t>
         </is>
       </c>
       <c r="I12" s="20" t="inlineStr">
@@ -3737,22 +3793,27 @@
           <t>Protection: Local Snapshots | Replication: None</t>
         </is>
       </c>
-      <c r="K12" s="33" t="inlineStr">
+      <c r="K12" s="20" t="inlineStr">
+        <is>
+          <t>Volumes CSV: Volume Set 'Production1' — Protection Level='Local Snapshots', Replication Type='None', Export Status=Exported. No DR replication target configured.</t>
+        </is>
+      </c>
+      <c r="L12" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L12" s="20" t="inlineStr">
-        <is>
-          <t>hai01p-mp</t>
-        </is>
-      </c>
       <c r="M12" s="20" t="inlineStr">
         <is>
+          <t>Volumes_Inventory_06092026_120519.csv: hai01p-mp</t>
+        </is>
+      </c>
+      <c r="N12" s="20" t="inlineStr">
+        <is>
           <t>Volume Set: Production1</t>
         </is>
       </c>
-      <c r="N12" s="20" t="inlineStr">
+      <c r="O12" s="20" t="inlineStr">
         <is>
           <t>SAN - No Volume Replication Configured</t>
         </is>
@@ -3786,7 +3847,7 @@
       <c r="G13" s="36" t="inlineStr"/>
       <c r="H13" s="21" t="inlineStr">
         <is>
-          <t>Volume set 'Production2' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
+          <t>No remote replication is configured for this exported volume set. Local snapshots alone cannot protect against site-level failure, storage hardware failure, or ransomware that corrupts all local snapshots before a recovery point is reached.</t>
         </is>
       </c>
       <c r="I13" s="21" t="inlineStr">
@@ -3799,22 +3860,27 @@
           <t>Protection: Local Snapshots | Replication: None</t>
         </is>
       </c>
-      <c r="K13" s="33" t="inlineStr">
+      <c r="K13" s="21" t="inlineStr">
+        <is>
+          <t>Volumes CSV: Volume Set 'Production2' — Protection Level='Local Snapshots', Replication Type='None', Export Status=Exported. No DR replication target configured.</t>
+        </is>
+      </c>
+      <c r="L13" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L13" s="21" t="inlineStr">
-        <is>
-          <t>hai01p-mp</t>
-        </is>
-      </c>
       <c r="M13" s="21" t="inlineStr">
         <is>
+          <t>Volumes_Inventory_06092026_120519.csv: hai01p-mp</t>
+        </is>
+      </c>
+      <c r="N13" s="21" t="inlineStr">
+        <is>
           <t>Volume Set: Production2</t>
         </is>
       </c>
-      <c r="N13" s="21" t="inlineStr">
+      <c r="O13" s="21" t="inlineStr">
         <is>
           <t>SAN - No Volume Replication Configured</t>
         </is>
@@ -3856,7 +3922,7 @@
       </c>
       <c r="H14" s="20" t="inlineStr">
         <is>
-          <t>No login warning banner (MOTD) is configured. The [Banner] section in configShow is empty. A legal notice banner is required by most compliance frameworks and establishes legal standing for access monitoring.</t>
+          <t>No login warning banner (MOTD) is configured on the switch. A legal notice banner is required by most compliance frameworks to establish legal standing for access monitoring and deter unauthorized use.</t>
         </is>
       </c>
       <c r="I14" s="20" t="inlineStr">
@@ -3869,22 +3935,27 @@
           <t>configShow line 377</t>
         </is>
       </c>
-      <c r="K14" s="33" t="inlineStr">
+      <c r="K14" s="20" t="inlineStr">
+        <is>
+          <t>configShow: [Banner] section is empty (line 377). No warning is presented to users at login.</t>
+        </is>
+      </c>
+      <c r="L14" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L14" s="20" t="inlineStr">
-        <is>
-          <t>swd77 (Domain 1)</t>
-        </is>
-      </c>
       <c r="M14" s="20" t="inlineStr">
         <is>
+          <t>Brocade01 2026-06-01.log: swd77 (Domain 1)</t>
+        </is>
+      </c>
+      <c r="N14" s="20" t="inlineStr">
+        <is>
           <t>[Banner] section empty (377)</t>
         </is>
       </c>
-      <c r="N14" s="20" t="inlineStr">
+      <c r="O14" s="20" t="inlineStr">
         <is>
           <t>SAN - No Login Banner Configured</t>
         </is>
@@ -3922,7 +3993,7 @@
       <c r="G15" s="36" t="inlineStr"/>
       <c r="H15" s="21" t="inlineStr">
         <is>
-          <t>4 zone(s) are defined but not included in any active zone configuration (cfg): z_EXCHANGE2_EVA2_A; z_SQLPROD2_EVA2_A; z_SQLPROD_EVA2_A; z_SQLTEST_EVA2_A. These may represent decommissioned hosts or legacy storage (e.g., EVA2 arrays) removed without zone cleanup. Stale zones inflate configuration and may be accidentally re-activated.</t>
+          <t>Zone definitions exist in the fabric that are not included in any active zone configuration. Orphaned zones may represent decommissioned hosts or storage removed without cleaning up the zone database, and can be accidentally re-activated.</t>
         </is>
       </c>
       <c r="I15" s="21" t="inlineStr">
@@ -3935,22 +4006,27 @@
           <t>z_EXCHANGE2_EVA2_A; z_SQLPROD2_EVA2_A; z_SQLPROD_EVA2_A; z_SQLTEST_EVA2_A</t>
         </is>
       </c>
-      <c r="K15" s="33" t="inlineStr">
+      <c r="K15" s="21" t="inlineStr">
+        <is>
+          <t>4 zone(s) defined but not in active cfg 'ZZZZZG_SAN_A': z_EXCHANGE2_EVA2_A; z_SQLPROD2_EVA2_A; z_SQLPROD_EVA2_A; z_SQLTEST_EVA2_A.</t>
+        </is>
+      </c>
+      <c r="L15" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L15" s="21" t="inlineStr">
-        <is>
-          <t>swd77 (Domain 1)</t>
-        </is>
-      </c>
       <c r="M15" s="21" t="inlineStr">
         <is>
+          <t>Brocade01 2026-06-01.log: swd77 (Domain 1)</t>
+        </is>
+      </c>
+      <c r="N15" s="21" t="inlineStr">
+        <is>
           <t>4 orphaned zone(s) (419)</t>
         </is>
       </c>
-      <c r="N15" s="21" t="inlineStr">
+      <c r="O15" s="21" t="inlineStr">
         <is>
           <t>SAN - Stale Zone Definitions</t>
         </is>
@@ -3992,7 +4068,7 @@
       </c>
       <c r="H16" s="20" t="inlineStr">
         <is>
-          <t>No login warning banner (MOTD) is configured. The [Banner] section in configShow is empty. A legal notice banner is required by most compliance frameworks and establishes legal standing for access monitoring.</t>
+          <t>No login warning banner (MOTD) is configured on the switch. A legal notice banner is required by most compliance frameworks to establish legal standing for access monitoring and deter unauthorized use.</t>
         </is>
       </c>
       <c r="I16" s="20" t="inlineStr">
@@ -4005,22 +4081,27 @@
           <t>configShow line 375</t>
         </is>
       </c>
-      <c r="K16" s="33" t="inlineStr">
+      <c r="K16" s="20" t="inlineStr">
+        <is>
+          <t>configShow: [Banner] section is empty (line 375). No warning is presented to users at login.</t>
+        </is>
+      </c>
+      <c r="L16" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L16" s="20" t="inlineStr">
-        <is>
-          <t>swd77 (Domain 2)</t>
-        </is>
-      </c>
       <c r="M16" s="20" t="inlineStr">
         <is>
+          <t>Brocade02 2026-06-01.log: swd77 (Domain 2)</t>
+        </is>
+      </c>
+      <c r="N16" s="20" t="inlineStr">
+        <is>
           <t>[Banner] section empty (375)</t>
         </is>
       </c>
-      <c r="N16" s="20" t="inlineStr">
+      <c r="O16" s="20" t="inlineStr">
         <is>
           <t>SAN - No Login Banner Configured</t>
         </is>
@@ -4058,7 +4139,7 @@
       <c r="G17" s="36" t="inlineStr"/>
       <c r="H17" s="21" t="inlineStr">
         <is>
-          <t>5 zone(s) are defined but not included in any active zone configuration (cfg): z_EXCHANGE2_EVA2_B; z_SQLPROD2_EVA2_B; z_SQLPROD_EVA2_B; z_SQLTEST2_EVA_B; z_SQLTEST_EVA_B. These may represent decommissioned hosts or legacy storage (e.g., EVA2 arrays) removed without zone cleanup. Stale zones inflate configuration and may be accidentally re-activated.</t>
+          <t>Zone definitions exist in the fabric that are not included in any active zone configuration. Orphaned zones may represent decommissioned hosts or storage removed without cleaning up the zone database, and can be accidentally re-activated.</t>
         </is>
       </c>
       <c r="I17" s="21" t="inlineStr">
@@ -4071,22 +4152,27 @@
           <t>z_EXCHANGE2_EVA2_B; z_SQLPROD2_EVA2_B; z_SQLPROD_EVA2_B; z_SQLTEST2_EVA_B; z_SQLTEST_EVA_B</t>
         </is>
       </c>
-      <c r="K17" s="33" t="inlineStr">
+      <c r="K17" s="21" t="inlineStr">
+        <is>
+          <t>5 zone(s) defined but not in active cfg 'ZZZZZG_SAN_B': z_EXCHANGE2_EVA2_B; z_SQLPROD2_EVA2_B; z_SQLPROD_EVA2_B; z_SQLTEST2_EVA_B; z_SQLTEST_EVA_B.</t>
+        </is>
+      </c>
+      <c r="L17" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L17" s="21" t="inlineStr">
-        <is>
-          <t>swd77 (Domain 2)</t>
-        </is>
-      </c>
       <c r="M17" s="21" t="inlineStr">
         <is>
+          <t>Brocade02 2026-06-01.log: swd77 (Domain 2)</t>
+        </is>
+      </c>
+      <c r="N17" s="21" t="inlineStr">
+        <is>
           <t>5 orphaned zone(s) (417)</t>
         </is>
       </c>
-      <c r="N17" s="21" t="inlineStr">
+      <c r="O17" s="21" t="inlineStr">
         <is>
           <t>SAN - Stale Zone Definitions</t>
         </is>
@@ -4120,7 +4206,7 @@
       <c r="G18" s="32" t="inlineStr"/>
       <c r="H18" s="20" t="inlineStr">
         <is>
-          <t>4 FC port(s) are in 'loss_sync' state: 0:3:2, 0:3:4, 1:3:2, 1:3:4. These ports have lost synchronization with their SAN fabric counterpart and are not passing traffic. This reduces path redundancy and may indicate a cabling, SFP, or switch-side fault.</t>
+          <t>One or more FC target ports are in 'loss_sync' state, indicating lost synchronization with the fabric. Degraded ports are not passing traffic, reducing path redundancy for connected hosts and indicating a potential hardware or cabling fault.</t>
         </is>
       </c>
       <c r="I18" s="20" t="inlineStr">
@@ -4133,22 +4219,27 @@
           <t>Ports in loss_sync: 0:3:2, 0:3:4, 1:3:2, 1:3:4</t>
         </is>
       </c>
-      <c r="K18" s="33" t="inlineStr">
+      <c r="K18" s="20" t="inlineStr">
+        <is>
+          <t>showport: 4 port(s) in loss_sync state: 0:3:2, 0:3:4, 1:3:2, 1:3:4. These ports have lost link-level synchronization with the connected Brocade switch and are not carrying I/O.</t>
+        </is>
+      </c>
+      <c r="L18" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L18" s="20" t="inlineStr">
-        <is>
-          <t>ZZZZZ01p-mp</t>
-        </is>
-      </c>
       <c r="M18" s="20" t="inlineStr">
         <is>
+          <t>Alletra 2026-06-09-01.log: ZZZZZ01p-mp</t>
+        </is>
+      </c>
+      <c r="N18" s="20" t="inlineStr">
+        <is>
           <t>loss_sync: 0:3:2, 0:3:4, 1:3:2, 1:3:4</t>
         </is>
       </c>
-      <c r="N18" s="20" t="inlineStr">
+      <c r="O18" s="20" t="inlineStr">
         <is>
           <t>SAN - Degraded FC Ports</t>
         </is>
@@ -4186,7 +4277,7 @@
       </c>
       <c r="H19" s="21" t="inlineStr">
         <is>
-          <t>The HP Alletra MP REST API (WSAPI) is enabled and active on HTTPS 443. The REST API exposes full array management including volume creation, deletion, VLUN mapping, and host definitions. Unauthorized access allows complete storage compromise without FC fabric access.</t>
+          <t>The array REST API (WSAPI) is enabled and active. The API exposes full array management capabilities including volume, host, and VLUN management without requiring FC fabric access to execute changes.</t>
         </is>
       </c>
       <c r="I19" s="21" t="inlineStr">
@@ -4199,22 +4290,27 @@
           <t>WSAPI: Enabled / Active, HTTPS 443</t>
         </is>
       </c>
-      <c r="K19" s="33" t="inlineStr">
+      <c r="K19" s="21" t="inlineStr">
+        <is>
+          <t>showwsapi: Service=Enabled, State=Active on HTTPS port 443. REST API is accessible and accepting connections.</t>
+        </is>
+      </c>
+      <c r="L19" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L19" s="21" t="inlineStr">
-        <is>
-          <t>ZZZZZ01p-mp</t>
-        </is>
-      </c>
       <c r="M19" s="21" t="inlineStr">
         <is>
+          <t>Alletra 2026-06-09-01.log: ZZZZZ01p-mp</t>
+        </is>
+      </c>
+      <c r="N19" s="21" t="inlineStr">
+        <is>
           <t>WSAPI: Enabled / Active on HTTPS 443</t>
         </is>
       </c>
-      <c r="N19" s="21" t="inlineStr">
+      <c r="O19" s="21" t="inlineStr">
         <is>
           <t>SAN - REST API Exposed</t>
         </is>
@@ -4248,7 +4344,7 @@
       <c r="G20" s="32" t="inlineStr"/>
       <c r="H20" s="20" t="inlineStr">
         <is>
-          <t>MAPS is using the default policy 'dflt_base_policy' rather than a customized environment-specific policy. Default thresholds may not match this fabric's traffic patterns, causing missed alerts or excessive noise.</t>
+          <t>MAPS (Monitoring and Alerting Policy Suite) is using the default monitoring policy rather than a customized environment-specific policy. Default thresholds may miss or over-alert on issues specific to this fabric.</t>
         </is>
       </c>
       <c r="I20" s="20" t="inlineStr">
@@ -4257,22 +4353,27 @@
         </is>
       </c>
       <c r="J20" s="20" t="inlineStr"/>
-      <c r="K20" s="33" t="inlineStr">
+      <c r="K20" s="20" t="inlineStr">
+        <is>
+          <t>configShow: maps.activePolicy=dflt_base_policy. Default policy thresholds not tuned to this environment's traffic patterns.</t>
+        </is>
+      </c>
+      <c r="L20" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L20" s="20" t="inlineStr">
-        <is>
-          <t>swd77 (Domain 1)</t>
-        </is>
-      </c>
       <c r="M20" s="20" t="inlineStr">
         <is>
+          <t>Brocade01 2026-06-01.log: swd77 (Domain 1)</t>
+        </is>
+      </c>
+      <c r="N20" s="20" t="inlineStr">
+        <is>
           <t>maps.activePolicy: dflt_base_policy</t>
         </is>
       </c>
-      <c r="N20" s="20" t="inlineStr">
+      <c r="O20" s="20" t="inlineStr">
         <is>
           <t>SAN - Default MAPS Monitoring Policy</t>
         </is>
@@ -4306,7 +4407,7 @@
       <c r="G21" s="36" t="inlineStr"/>
       <c r="H21" s="21" t="inlineStr">
         <is>
-          <t>MAPS is using the default policy 'dflt_base_policy' rather than a customized environment-specific policy. Default thresholds may not match this fabric's traffic patterns, causing missed alerts or excessive noise.</t>
+          <t>MAPS (Monitoring and Alerting Policy Suite) is using the default monitoring policy rather than a customized environment-specific policy. Default thresholds may miss or over-alert on issues specific to this fabric.</t>
         </is>
       </c>
       <c r="I21" s="21" t="inlineStr">
@@ -4315,22 +4416,27 @@
         </is>
       </c>
       <c r="J21" s="21" t="inlineStr"/>
-      <c r="K21" s="33" t="inlineStr">
+      <c r="K21" s="21" t="inlineStr">
+        <is>
+          <t>configShow: maps.activePolicy=dflt_base_policy. Default policy thresholds not tuned to this environment's traffic patterns.</t>
+        </is>
+      </c>
+      <c r="L21" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L21" s="21" t="inlineStr">
-        <is>
-          <t>swd77 (Domain 2)</t>
-        </is>
-      </c>
       <c r="M21" s="21" t="inlineStr">
         <is>
+          <t>Brocade02 2026-06-01.log: swd77 (Domain 2)</t>
+        </is>
+      </c>
+      <c r="N21" s="21" t="inlineStr">
+        <is>
           <t>maps.activePolicy: dflt_base_policy</t>
         </is>
       </c>
-      <c r="N21" s="21" t="inlineStr">
+      <c r="O21" s="21" t="inlineStr">
         <is>
           <t>SAN - Default MAPS Monitoring Policy</t>
         </is>
@@ -4364,7 +4470,7 @@
       <c r="G22" s="32" t="inlineStr"/>
       <c r="H22" s="20" t="inlineStr">
         <is>
-          <t>5 FC storage device(s) have 'Perennially Reserved' = 'No'. For FC LUNs not consumed as VMFS datastores on this host, this causes unnecessary SCSI reservation probes and path thrashing at host boot.</t>
+          <t>FC storage devices presented to ESXi hosts do not have 'Perennially Reserved' enabled. For FC LUNs not actively consumed as VMFS datastores, this causes unnecessary SCSI reservation probes and potential path thrashing at ESXi host boot.</t>
         </is>
       </c>
       <c r="I22" s="20" t="inlineStr">
@@ -4377,29 +4483,34 @@
           <t>naa.60002ac0000000000000002b0002e9bd; naa.60002ac0000000000000002c0002e9bd; naa.60002ac0000000000000002e0002e9bd; naa.60002ac000000000000000130002e9bd; naa.60002ac0000000000000002d0002e9bd</t>
         </is>
       </c>
-      <c r="K22" s="33" t="inlineStr">
+      <c r="K22" s="20" t="inlineStr">
+        <is>
+          <t>storage-devices-export-data.csv: 5 FC disk(s) with Perennially Reserved=No: naa.60002ac0000000000000002b0002e9bd; naa.60002ac0000000000000002c0002e9bd; naa.60002ac0000000000000002e0002e9bd; naa.60002ac000000000000000130002e9bd; naa.60002ac0000000000000002d0002e9bd. ESXi will probe these LUNs for SCSI reservations on every boot.</t>
+        </is>
+      </c>
+      <c r="L22" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L22" s="20" t="inlineStr">
-        <is>
-          <t>VMware ESXi</t>
-        </is>
-      </c>
       <c r="M22" s="20" t="inlineStr">
         <is>
+          <t>storage-devices-export-data.csv: VMware ESXi</t>
+        </is>
+      </c>
+      <c r="N22" s="20" t="inlineStr">
+        <is>
           <t>5 FC disk(s)</t>
         </is>
       </c>
-      <c r="N22" s="20" t="inlineStr">
+      <c r="O22" s="20" t="inlineStr">
         <is>
           <t>SAN - Perennially Reserved Not Configured</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N1"/>
+  <autoFilter ref="A1:O1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4493,7 +4604,7 @@
       <c r="D6" s="40" t="inlineStr"/>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>No CHAP authentication is configured for 5 ESX host(s): ESX02, ESX04, ESX05, ESX06, ESX07. Both Initiator CHAP and Target CHAP show '--' in 'showhost -chap'. Without CHAP, any host presenting the correct WWN can authenticate to the array. In a compromised or miscabled environment this allows unauthorized LUN access.</t>
+          <t>No CHAP (Challenge-Handshake Authentication Protocol) authentication is configured for storage hosts. Without CHAP, any host presenting the correct WWN can authenticate to the array, enabling unauthorized LUN access in a compromised or miscabled environment.</t>
         </is>
       </c>
       <c r="F6" s="20" t="inlineStr">
@@ -4521,7 +4632,7 @@
       <c r="D7" s="41" t="inlineStr"/>
       <c r="E7" s="21" t="inlineStr">
         <is>
-          <t>No SSH public keys are configured on the Alletra MP. Administrative access relies exclusively on password authentication. Password-only authentication is weaker than key-based auth and does not meet PCI DSS requirements for strong cryptographic access controls.</t>
+          <t>No SSH public keys are configured on the storage array. Administrative access relies exclusively on password authentication, which does not meet requirements for strong cryptographic access controls.</t>
         </is>
       </c>
       <c r="F7" s="21" t="inlineStr">
@@ -4588,7 +4699,7 @@
       <c r="D11" s="41" t="inlineStr"/>
       <c r="E11" s="21" t="inlineStr">
         <is>
-          <t>The following security baseline commands returned 'invalid command name' on this firmware version: showpasswordpolicy, showsnmp, showsyslog, showaudit, showtime. Password policy, SNMP configuration, syslog/audit logging, and time synchronization cannot be verified from the CLI, leaving key security controls in an unknown compliance state.</t>
+          <t>Security baseline commands are not available on this firmware version. Password policy, SNMP configuration, syslog, audit logging, and time synchronization settings cannot be verified from the CLI, leaving key security controls in an unknown compliance state.</t>
         </is>
       </c>
       <c r="F11" s="21" t="inlineStr">
@@ -4620,7 +4731,7 @@
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
-          <t>No login warning banner (MOTD) is configured. The [Banner] section in configShow is empty. A legal notice banner is required by most compliance frameworks and establishes legal standing for access monitoring.</t>
+          <t>No login warning banner (MOTD) is configured on the switch. A legal notice banner is required by most compliance frameworks to establish legal standing for access monitoring and deter unauthorized use.</t>
         </is>
       </c>
       <c r="F12" s="20" t="inlineStr">
@@ -4652,7 +4763,7 @@
       </c>
       <c r="E13" s="21" t="inlineStr">
         <is>
-          <t>No login warning banner (MOTD) is configured. The [Banner] section in configShow is empty. A legal notice banner is required by most compliance frameworks and establishes legal standing for access monitoring.</t>
+          <t>No login warning banner (MOTD) is configured on the switch. A legal notice banner is required by most compliance frameworks to establish legal standing for access monitoring and deter unauthorized use.</t>
         </is>
       </c>
       <c r="F13" s="21" t="inlineStr">
@@ -4719,7 +4830,7 @@
       <c r="D17" s="41" t="inlineStr"/>
       <c r="E17" s="21" t="inlineStr">
         <is>
-          <t>The HP Alletra MP REST API (WSAPI) is enabled and active on HTTPS 443. The REST API exposes full array management including volume creation, deletion, VLUN mapping, and host definitions. Unauthorized access allows complete storage compromise without FC fabric access.</t>
+          <t>The array REST API (WSAPI) is enabled and active. The API exposes full array management capabilities including volume, host, and VLUN management without requiring FC fabric access to execute changes.</t>
         </is>
       </c>
       <c r="F17" s="21" t="inlineStr">
@@ -4800,7 +4911,7 @@
       <c r="D24" s="40" t="inlineStr"/>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>The following security baseline commands returned 'invalid command name' on this firmware version: showpasswordpolicy, showsnmp, showsyslog, showaudit, showtime. Password policy, SNMP configuration, syslog/audit logging, and time synchronization cannot be verified from the CLI, leaving key security controls in an unknown compliance state.</t>
+          <t>Security baseline commands are not available on this firmware version. Password policy, SNMP configuration, syslog, audit logging, and time synchronization settings cannot be verified from the CLI, leaving key security controls in an unknown compliance state.</t>
         </is>
       </c>
       <c r="F24" s="20" t="inlineStr">
@@ -4828,7 +4939,7 @@
       <c r="D25" s="41" t="inlineStr"/>
       <c r="E25" s="21" t="inlineStr">
         <is>
-          <t>MAPS is using the default policy 'dflt_base_policy' rather than a customized environment-specific policy. Default thresholds may not match this fabric's traffic patterns, causing missed alerts or excessive noise.</t>
+          <t>MAPS (Monitoring and Alerting Policy Suite) is using the default monitoring policy rather than a customized environment-specific policy. Default thresholds may miss or over-alert on issues specific to this fabric.</t>
         </is>
       </c>
       <c r="F25" s="21" t="inlineStr">
@@ -4856,7 +4967,7 @@
       <c r="D26" s="40" t="inlineStr"/>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>MAPS is using the default policy 'dflt_base_policy' rather than a customized environment-specific policy. Default thresholds may not match this fabric's traffic patterns, causing missed alerts or excessive noise.</t>
+          <t>MAPS (Monitoring and Alerting Policy Suite) is using the default monitoring policy rather than a customized environment-specific policy. Default thresholds may miss or over-alert on issues specific to this fabric.</t>
         </is>
       </c>
       <c r="F26" s="20" t="inlineStr">
@@ -4937,7 +5048,7 @@
       <c r="D33" s="41" t="inlineStr"/>
       <c r="E33" s="21" t="inlineStr">
         <is>
-          <t>Volume set 'DevTest1' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
+          <t>No remote replication is configured for this exported volume set. Local snapshots alone cannot protect against site-level failure, storage hardware failure, or ransomware that corrupts all local snapshots before a recovery point is reached.</t>
         </is>
       </c>
       <c r="F33" s="21" t="inlineStr">
@@ -4965,7 +5076,7 @@
       <c r="D34" s="40" t="inlineStr"/>
       <c r="E34" s="20" t="inlineStr">
         <is>
-          <t>Volume set 'Infrastructure1' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
+          <t>No remote replication is configured for this exported volume set. Local snapshots alone cannot protect against site-level failure, storage hardware failure, or ransomware that corrupts all local snapshots before a recovery point is reached.</t>
         </is>
       </c>
       <c r="F34" s="20" t="inlineStr">
@@ -4993,7 +5104,7 @@
       <c r="D35" s="41" t="inlineStr"/>
       <c r="E35" s="21" t="inlineStr">
         <is>
-          <t>Volume set 'Infrastructure2' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
+          <t>No remote replication is configured for this exported volume set. Local snapshots alone cannot protect against site-level failure, storage hardware failure, or ransomware that corrupts all local snapshots before a recovery point is reached.</t>
         </is>
       </c>
       <c r="F35" s="21" t="inlineStr">
@@ -5021,7 +5132,7 @@
       <c r="D36" s="40" t="inlineStr"/>
       <c r="E36" s="20" t="inlineStr">
         <is>
-          <t>Volume set 'Production1' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
+          <t>No remote replication is configured for this exported volume set. Local snapshots alone cannot protect against site-level failure, storage hardware failure, or ransomware that corrupts all local snapshots before a recovery point is reached.</t>
         </is>
       </c>
       <c r="F36" s="20" t="inlineStr">
@@ -5049,7 +5160,7 @@
       <c r="D37" s="41" t="inlineStr"/>
       <c r="E37" s="21" t="inlineStr">
         <is>
-          <t>Volume set 'Production2' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
+          <t>No remote replication is configured for this exported volume set. Local snapshots alone cannot protect against site-level failure, storage hardware failure, or ransomware that corrupts all local snapshots before a recovery point is reached.</t>
         </is>
       </c>
       <c r="F37" s="21" t="inlineStr">
@@ -5116,7 +5227,7 @@
       <c r="D41" s="41" t="inlineStr"/>
       <c r="E41" s="21" t="inlineStr">
         <is>
-          <t>Volume set 'DevTest1' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
+          <t>No remote replication is configured for this exported volume set. Local snapshots alone cannot protect against site-level failure, storage hardware failure, or ransomware that corrupts all local snapshots before a recovery point is reached.</t>
         </is>
       </c>
       <c r="F41" s="21" t="inlineStr">
@@ -5144,7 +5255,7 @@
       <c r="D42" s="40" t="inlineStr"/>
       <c r="E42" s="20" t="inlineStr">
         <is>
-          <t>Volume set 'Infrastructure1' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
+          <t>No remote replication is configured for this exported volume set. Local snapshots alone cannot protect against site-level failure, storage hardware failure, or ransomware that corrupts all local snapshots before a recovery point is reached.</t>
         </is>
       </c>
       <c r="F42" s="20" t="inlineStr">
@@ -5172,7 +5283,7 @@
       <c r="D43" s="41" t="inlineStr"/>
       <c r="E43" s="21" t="inlineStr">
         <is>
-          <t>Volume set 'Infrastructure2' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
+          <t>No remote replication is configured for this exported volume set. Local snapshots alone cannot protect against site-level failure, storage hardware failure, or ransomware that corrupts all local snapshots before a recovery point is reached.</t>
         </is>
       </c>
       <c r="F43" s="21" t="inlineStr">
@@ -5200,7 +5311,7 @@
       <c r="D44" s="40" t="inlineStr"/>
       <c r="E44" s="20" t="inlineStr">
         <is>
-          <t>Volume set 'Production1' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
+          <t>No remote replication is configured for this exported volume set. Local snapshots alone cannot protect against site-level failure, storage hardware failure, or ransomware that corrupts all local snapshots before a recovery point is reached.</t>
         </is>
       </c>
       <c r="F44" s="20" t="inlineStr">
@@ -5228,7 +5339,7 @@
       <c r="D45" s="41" t="inlineStr"/>
       <c r="E45" s="21" t="inlineStr">
         <is>
-          <t>Volume set 'Production2' is exported to production hosts with Protection Level 'Local Snapshots' and Replication Type 'None'. No remote replication is configured. Local snapshots alone cannot protect against a site-level failure, storage hardware failure, or ransomware that corrupts all snapshots.</t>
+          <t>No remote replication is configured for this exported volume set. Local snapshots alone cannot protect against site-level failure, storage hardware failure, or ransomware that corrupts all local snapshots before a recovery point is reached.</t>
         </is>
       </c>
       <c r="F45" s="21" t="inlineStr">
@@ -5299,7 +5410,7 @@
       </c>
       <c r="E49" s="21" t="inlineStr">
         <is>
-          <t>FC Authentication Policy is disabled (auth.policy=0). No DH-CHAP authentication is required between fabric ports. An unauthorized switch or rogue HBA can join the fabric without credentials, enabling eavesdropping and spoofed SCSI commands on VMware datastores.</t>
+          <t>FC Authentication Policy (DH-CHAP) is disabled. No authentication is required between fabric ports, allowing unauthorized switches or rogue HBAs to join the fabric without credentials and enabling fabric eavesdropping and spoofed SCSI commands.</t>
         </is>
       </c>
       <c r="F49" s="21" t="inlineStr">
@@ -5331,7 +5442,7 @@
       </c>
       <c r="E50" s="20" t="inlineStr">
         <is>
-          <t>The default zone is set to 'allaccess'. Any device not placed in a named zone can communicate with ALL other unzoned devices, creating an open fabric. A rogue HBA inserted into any open port gains full fabric visibility. This violates SAN isolation requirements for VMware.</t>
+          <t>The default zone policy is set to 'allaccess'. Devices not placed in a named zone can communicate with all other unzoned devices, creating an open fabric with no isolation between initiators and targets.</t>
         </is>
       </c>
       <c r="F50" s="20" t="inlineStr">
@@ -5363,7 +5474,7 @@
       </c>
       <c r="E51" s="21" t="inlineStr">
         <is>
-          <t>FC Authentication Policy is disabled (auth.policy=0). No DH-CHAP authentication is required between fabric ports. An unauthorized switch or rogue HBA can join the fabric without credentials, enabling eavesdropping and spoofed SCSI commands on VMware datastores.</t>
+          <t>FC Authentication Policy (DH-CHAP) is disabled. No authentication is required between fabric ports, allowing unauthorized switches or rogue HBAs to join the fabric without credentials and enabling fabric eavesdropping and spoofed SCSI commands.</t>
         </is>
       </c>
       <c r="F51" s="21" t="inlineStr">
@@ -5395,7 +5506,7 @@
       </c>
       <c r="E52" s="20" t="inlineStr">
         <is>
-          <t>The default zone is set to 'allaccess'. Any device not placed in a named zone can communicate with ALL other unzoned devices, creating an open fabric. A rogue HBA inserted into any open port gains full fabric visibility. This violates SAN isolation requirements for VMware.</t>
+          <t>The default zone policy is set to 'allaccess'. Devices not placed in a named zone can communicate with all other unzoned devices, creating an open fabric with no isolation between initiators and targets.</t>
         </is>
       </c>
       <c r="F52" s="20" t="inlineStr">
@@ -5423,7 +5534,7 @@
       <c r="D53" s="41" t="inlineStr"/>
       <c r="E53" s="21" t="inlineStr">
         <is>
-          <t>No CHAP authentication is configured for 5 ESX host(s): ESX02, ESX04, ESX05, ESX06, ESX07. Both Initiator CHAP and Target CHAP show '--' in 'showhost -chap'. Without CHAP, any host presenting the correct WWN can authenticate to the array. In a compromised or miscabled environment this allows unauthorized LUN access.</t>
+          <t>No CHAP (Challenge-Handshake Authentication Protocol) authentication is configured for storage hosts. Without CHAP, any host presenting the correct WWN can authenticate to the array, enabling unauthorized LUN access in a compromised or miscabled environment.</t>
         </is>
       </c>
       <c r="F53" s="21" t="inlineStr">
@@ -5455,7 +5566,7 @@
       </c>
       <c r="E54" s="20" t="inlineStr">
         <is>
-          <t>4 zone(s) are defined but not included in any active zone configuration (cfg): z_EXCHANGE2_EVA2_A; z_SQLPROD2_EVA2_A; z_SQLPROD_EVA2_A; z_SQLTEST_EVA2_A. These may represent decommissioned hosts or legacy storage (e.g., EVA2 arrays) removed without zone cleanup. Stale zones inflate configuration and may be accidentally re-activated.</t>
+          <t>Zone definitions exist in the fabric that are not included in any active zone configuration. Orphaned zones may represent decommissioned hosts or storage removed without cleaning up the zone database, and can be accidentally re-activated.</t>
         </is>
       </c>
       <c r="F54" s="20" t="inlineStr">
@@ -5487,7 +5598,7 @@
       </c>
       <c r="E55" s="21" t="inlineStr">
         <is>
-          <t>5 zone(s) are defined but not included in any active zone configuration (cfg): z_EXCHANGE2_EVA2_B; z_SQLPROD2_EVA2_B; z_SQLPROD_EVA2_B; z_SQLTEST2_EVA_B; z_SQLTEST_EVA_B. These may represent decommissioned hosts or legacy storage (e.g., EVA2 arrays) removed without zone cleanup. Stale zones inflate configuration and may be accidentally re-activated.</t>
+          <t>Zone definitions exist in the fabric that are not included in any active zone configuration. Orphaned zones may represent decommissioned hosts or storage removed without cleaning up the zone database, and can be accidentally re-activated.</t>
         </is>
       </c>
       <c r="F55" s="21" t="inlineStr">
@@ -5515,7 +5626,7 @@
       <c r="D56" s="40" t="inlineStr"/>
       <c r="E56" s="20" t="inlineStr">
         <is>
-          <t>4 FC port(s) are in 'loss_sync' state: 0:3:2, 0:3:4, 1:3:2, 1:3:4. These ports have lost synchronization with their SAN fabric counterpart and are not passing traffic. This reduces path redundancy and may indicate a cabling, SFP, or switch-side fault.</t>
+          <t>One or more FC target ports are in 'loss_sync' state, indicating lost synchronization with the fabric. Degraded ports are not passing traffic, reducing path redundancy for connected hosts and indicating a potential hardware or cabling fault.</t>
         </is>
       </c>
       <c r="F56" s="20" t="inlineStr">
@@ -5543,7 +5654,7 @@
       <c r="D57" s="41" t="inlineStr"/>
       <c r="E57" s="21" t="inlineStr">
         <is>
-          <t>5 FC storage device(s) have 'Perennially Reserved' = 'No'. For FC LUNs not consumed as VMFS datastores on this host, this causes unnecessary SCSI reservation probes and path thrashing at host boot.</t>
+          <t>FC storage devices presented to ESXi hosts do not have 'Perennially Reserved' enabled. For FC LUNs not actively consumed as VMFS datastores, this causes unnecessary SCSI reservation probes and potential path thrashing at ESXi host boot.</t>
         </is>
       </c>
       <c r="F57" s="21" t="inlineStr">
@@ -5614,7 +5725,7 @@
       </c>
       <c r="E61" s="21" t="inlineStr">
         <is>
-          <t>FC Authentication Policy is disabled (auth.policy=0). No DH-CHAP authentication is required between fabric ports. An unauthorized switch or rogue HBA can join the fabric without credentials, enabling eavesdropping and spoofed SCSI commands on VMware datastores.</t>
+          <t>FC Authentication Policy (DH-CHAP) is disabled. No authentication is required between fabric ports, allowing unauthorized switches or rogue HBAs to join the fabric without credentials and enabling fabric eavesdropping and spoofed SCSI commands.</t>
         </is>
       </c>
       <c r="F61" s="21" t="inlineStr">
@@ -5646,7 +5757,7 @@
       </c>
       <c r="E62" s="20" t="inlineStr">
         <is>
-          <t>FC Authentication Policy is disabled (auth.policy=0). No DH-CHAP authentication is required between fabric ports. An unauthorized switch or rogue HBA can join the fabric without credentials, enabling eavesdropping and spoofed SCSI commands on VMware datastores.</t>
+          <t>FC Authentication Policy (DH-CHAP) is disabled. No authentication is required between fabric ports, allowing unauthorized switches or rogue HBAs to join the fabric without credentials and enabling fabric eavesdropping and spoofed SCSI commands.</t>
         </is>
       </c>
       <c r="F62" s="20" t="inlineStr">
@@ -5674,7 +5785,7 @@
       <c r="D63" s="41" t="inlineStr"/>
       <c r="E63" s="21" t="inlineStr">
         <is>
-          <t>The HP Alletra MP REST API (WSAPI) is enabled and active on HTTPS 443. The REST API exposes full array management including volume creation, deletion, VLUN mapping, and host definitions. Unauthorized access allows complete storage compromise without FC fabric access.</t>
+          <t>The array REST API (WSAPI) is enabled and active. The API exposes full array management capabilities including volume, host, and VLUN management without requiring FC fabric access to execute changes.</t>
         </is>
       </c>
       <c r="F63" s="21" t="inlineStr">
@@ -5741,7 +5852,7 @@
       <c r="D67" s="41" t="inlineStr"/>
       <c r="E67" s="21" t="inlineStr">
         <is>
-          <t>No SSH public keys are configured on the Alletra MP. Administrative access relies exclusively on password authentication. Password-only authentication is weaker than key-based auth and does not meet PCI DSS requirements for strong cryptographic access controls.</t>
+          <t>No SSH public keys are configured on the storage array. Administrative access relies exclusively on password authentication, which does not meet requirements for strong cryptographic access controls.</t>
         </is>
       </c>
       <c r="F67" s="21" t="inlineStr">
@@ -5812,7 +5923,7 @@
       </c>
       <c r="E71" s="21" t="inlineStr">
         <is>
-          <t>The default zone is set to 'allaccess'. Any device not placed in a named zone can communicate with ALL other unzoned devices, creating an open fabric. A rogue HBA inserted into any open port gains full fabric visibility. This violates SAN isolation requirements for VMware.</t>
+          <t>The default zone policy is set to 'allaccess'. Devices not placed in a named zone can communicate with all other unzoned devices, creating an open fabric with no isolation between initiators and targets.</t>
         </is>
       </c>
       <c r="F71" s="21" t="inlineStr">
@@ -5844,7 +5955,7 @@
       </c>
       <c r="E72" s="20" t="inlineStr">
         <is>
-          <t>The default zone is set to 'allaccess'. Any device not placed in a named zone can communicate with ALL other unzoned devices, creating an open fabric. A rogue HBA inserted into any open port gains full fabric visibility. This violates SAN isolation requirements for VMware.</t>
+          <t>The default zone policy is set to 'allaccess'. Devices not placed in a named zone can communicate with all other unzoned devices, creating an open fabric with no isolation between initiators and targets.</t>
         </is>
       </c>
       <c r="F72" s="20" t="inlineStr">
@@ -5969,7 +6080,7 @@
       </c>
       <c r="E5" s="21" t="inlineStr">
         <is>
-          <t>FC Authentication Policy is disabled (auth.policy=0). No DH-CHAP authentication is required between fabric ports. An unauthorized switch or rogue HBA can join the fabric without credentials, enabling eavesdropping and spoofed SCSI commands on VMware datastores.</t>
+          <t>FC Authentication Policy (DH-CHAP) is disabled. No authentication is required between fabric ports, allowing unauthorized switches or rogue HBAs to join the fabric without credentials and enabling fabric eavesdropping and spoofed SCSI commands.</t>
         </is>
       </c>
       <c r="F5" s="21" t="inlineStr">
@@ -6001,7 +6112,7 @@
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>The default zone is set to 'allaccess'. Any device not placed in a named zone can communicate with ALL other unzoned devices, creating an open fabric. A rogue HBA inserted into any open port gains full fabric visibility. This violates SAN isolation requirements for VMware.</t>
+          <t>The default zone policy is set to 'allaccess'. Devices not placed in a named zone can communicate with all other unzoned devices, creating an open fabric with no isolation between initiators and targets.</t>
         </is>
       </c>
       <c r="F6" s="20" t="inlineStr">
@@ -6033,7 +6144,7 @@
       </c>
       <c r="E7" s="21" t="inlineStr">
         <is>
-          <t>FC Authentication Policy is disabled (auth.policy=0). No DH-CHAP authentication is required between fabric ports. An unauthorized switch or rogue HBA can join the fabric without credentials, enabling eavesdropping and spoofed SCSI commands on VMware datastores.</t>
+          <t>FC Authentication Policy (DH-CHAP) is disabled. No authentication is required between fabric ports, allowing unauthorized switches or rogue HBAs to join the fabric without credentials and enabling fabric eavesdropping and spoofed SCSI commands.</t>
         </is>
       </c>
       <c r="F7" s="21" t="inlineStr">
@@ -6065,7 +6176,7 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>The default zone is set to 'allaccess'. Any device not placed in a named zone can communicate with ALL other unzoned devices, creating an open fabric. A rogue HBA inserted into any open port gains full fabric visibility. This violates SAN isolation requirements for VMware.</t>
+          <t>The default zone policy is set to 'allaccess'. Devices not placed in a named zone can communicate with all other unzoned devices, creating an open fabric with no isolation between initiators and targets.</t>
         </is>
       </c>
       <c r="F8" s="20" t="inlineStr">
@@ -6093,7 +6204,7 @@
       <c r="D9" s="41" t="inlineStr"/>
       <c r="E9" s="21" t="inlineStr">
         <is>
-          <t>No CHAP authentication is configured for 5 ESX host(s): ESX02, ESX04, ESX05, ESX06, ESX07. Both Initiator CHAP and Target CHAP show '--' in 'showhost -chap'. Without CHAP, any host presenting the correct WWN can authenticate to the array. In a compromised or miscabled environment this allows unauthorized LUN access.</t>
+          <t>No CHAP (Challenge-Handshake Authentication Protocol) authentication is configured for storage hosts. Without CHAP, any host presenting the correct WWN can authenticate to the array, enabling unauthorized LUN access in a compromised or miscabled environment.</t>
         </is>
       </c>
       <c r="F9" s="21" t="inlineStr">
@@ -6164,7 +6275,7 @@
       </c>
       <c r="E13" s="21" t="inlineStr">
         <is>
-          <t>The default zone is set to 'allaccess'. Any device not placed in a named zone can communicate with ALL other unzoned devices, creating an open fabric. A rogue HBA inserted into any open port gains full fabric visibility. This violates SAN isolation requirements for VMware.</t>
+          <t>The default zone policy is set to 'allaccess'. Devices not placed in a named zone can communicate with all other unzoned devices, creating an open fabric with no isolation between initiators and targets.</t>
         </is>
       </c>
       <c r="F13" s="21" t="inlineStr">
@@ -6196,7 +6307,7 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>The default zone is set to 'allaccess'. Any device not placed in a named zone can communicate with ALL other unzoned devices, creating an open fabric. A rogue HBA inserted into any open port gains full fabric visibility. This violates SAN isolation requirements for VMware.</t>
+          <t>The default zone policy is set to 'allaccess'. Devices not placed in a named zone can communicate with all other unzoned devices, creating an open fabric with no isolation between initiators and targets.</t>
         </is>
       </c>
       <c r="F14" s="20" t="inlineStr">
@@ -6263,7 +6374,7 @@
       <c r="D18" s="40" t="inlineStr"/>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>The following security baseline commands returned 'invalid command name' on this firmware version: showpasswordpolicy, showsnmp, showsyslog, showaudit, showtime. Password policy, SNMP configuration, syslog/audit logging, and time synchronization cannot be verified from the CLI, leaving key security controls in an unknown compliance state.</t>
+          <t>Security baseline commands are not available on this firmware version. Password policy, SNMP configuration, syslog, audit logging, and time synchronization settings cannot be verified from the CLI, leaving key security controls in an unknown compliance state.</t>
         </is>
       </c>
       <c r="F18" s="20" t="inlineStr">
@@ -6295,7 +6406,7 @@
       </c>
       <c r="E19" s="21" t="inlineStr">
         <is>
-          <t>No login warning banner (MOTD) is configured. The [Banner] section in configShow is empty. A legal notice banner is required by most compliance frameworks and establishes legal standing for access monitoring.</t>
+          <t>No login warning banner (MOTD) is configured on the switch. A legal notice banner is required by most compliance frameworks to establish legal standing for access monitoring and deter unauthorized use.</t>
         </is>
       </c>
       <c r="F19" s="21" t="inlineStr">
@@ -6327,7 +6438,7 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>No login warning banner (MOTD) is configured. The [Banner] section in configShow is empty. A legal notice banner is required by most compliance frameworks and establishes legal standing for access monitoring.</t>
+          <t>No login warning banner (MOTD) is configured on the switch. A legal notice banner is required by most compliance frameworks to establish legal standing for access monitoring and deter unauthorized use.</t>
         </is>
       </c>
       <c r="F20" s="20" t="inlineStr">
@@ -6394,7 +6505,7 @@
       <c r="D24" s="40" t="inlineStr"/>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>The HP Alletra MP REST API (WSAPI) is enabled and active on HTTPS 443. The REST API exposes full array management including volume creation, deletion, VLUN mapping, and host definitions. Unauthorized access allows complete storage compromise without FC fabric access.</t>
+          <t>The array REST API (WSAPI) is enabled and active. The API exposes full array management capabilities including volume, host, and VLUN management without requiring FC fabric access to execute changes.</t>
         </is>
       </c>
       <c r="F24" s="20" t="inlineStr">
@@ -6461,7 +6572,7 @@
       <c r="D28" s="40" t="inlineStr"/>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>No SSH public keys are configured on the Alletra MP. Administrative access relies exclusively on password authentication. Password-only authentication is weaker than key-based auth and does not meet PCI DSS requirements for strong cryptographic access controls.</t>
+          <t>No SSH public keys are configured on the storage array. Administrative access relies exclusively on password authentication, which does not meet requirements for strong cryptographic access controls.</t>
         </is>
       </c>
       <c r="F28" s="20" t="inlineStr">
@@ -6532,7 +6643,7 @@
       </c>
       <c r="E32" s="20" t="inlineStr">
         <is>
-          <t>FC Authentication Policy is disabled (auth.policy=0). No DH-CHAP authentication is required between fabric ports. An unauthorized switch or rogue HBA can join the fabric without credentials, enabling eavesdropping and spoofed SCSI commands on VMware datastores.</t>
+          <t>FC Authentication Policy (DH-CHAP) is disabled. No authentication is required between fabric ports, allowing unauthorized switches or rogue HBAs to join the fabric without credentials and enabling fabric eavesdropping and spoofed SCSI commands.</t>
         </is>
       </c>
       <c r="F32" s="20" t="inlineStr">
@@ -6564,7 +6675,7 @@
       </c>
       <c r="E33" s="21" t="inlineStr">
         <is>
-          <t>FC Authentication Policy is disabled (auth.policy=0). No DH-CHAP authentication is required between fabric ports. An unauthorized switch or rogue HBA can join the fabric without credentials, enabling eavesdropping and spoofed SCSI commands on VMware datastores.</t>
+          <t>FC Authentication Policy (DH-CHAP) is disabled. No authentication is required between fabric ports, allowing unauthorized switches or rogue HBAs to join the fabric without credentials and enabling fabric eavesdropping and spoofed SCSI commands.</t>
         </is>
       </c>
       <c r="F33" s="21" t="inlineStr">
@@ -6592,7 +6703,7 @@
       <c r="D34" s="40" t="inlineStr"/>
       <c r="E34" s="20" t="inlineStr">
         <is>
-          <t>No CHAP authentication is configured for 5 ESX host(s): ESX02, ESX04, ESX05, ESX06, ESX07. Both Initiator CHAP and Target CHAP show '--' in 'showhost -chap'. Without CHAP, any host presenting the correct WWN can authenticate to the array. In a compromised or miscabled environment this allows unauthorized LUN access.</t>
+          <t>No CHAP (Challenge-Handshake Authentication Protocol) authentication is configured for storage hosts. Without CHAP, any host presenting the correct WWN can authenticate to the array, enabling unauthorized LUN access in a compromised or miscabled environment.</t>
         </is>
       </c>
       <c r="F34" s="20" t="inlineStr">
@@ -6620,7 +6731,7 @@
       <c r="D35" s="41" t="inlineStr"/>
       <c r="E35" s="21" t="inlineStr">
         <is>
-          <t>No SSH public keys are configured on the Alletra MP. Administrative access relies exclusively on password authentication. Password-only authentication is weaker than key-based auth and does not meet PCI DSS requirements for strong cryptographic access controls.</t>
+          <t>No SSH public keys are configured on the storage array. Administrative access relies exclusively on password authentication, which does not meet requirements for strong cryptographic access controls.</t>
         </is>
       </c>
       <c r="F35" s="21" t="inlineStr">
@@ -6687,7 +6798,7 @@
       <c r="D39" s="41" t="inlineStr"/>
       <c r="E39" s="21" t="inlineStr">
         <is>
-          <t>The following security baseline commands returned 'invalid command name' on this firmware version: showpasswordpolicy, showsnmp, showsyslog, showaudit, showtime. Password policy, SNMP configuration, syslog/audit logging, and time synchronization cannot be verified from the CLI, leaving key security controls in an unknown compliance state.</t>
+          <t>Security baseline commands are not available on this firmware version. Password policy, SNMP configuration, syslog, audit logging, and time synchronization settings cannot be verified from the CLI, leaving key security controls in an unknown compliance state.</t>
         </is>
       </c>
       <c r="F39" s="21" t="inlineStr">

</xml_diff>

<commit_message>
Split filename out of Asset into new Source column
Asset now shows device name only; new Source column holds the filename
the finding came from.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/san/sample-san_analysis.xlsx
+++ b/san/sample-san_analysis.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCI DSS Mapping" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Security Issues'!$A$1:$O$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Security Issues'!$A$1:$P$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -762,7 +762,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-15 23:08:36    Switches: swd77 Domain 1; swd77 Domain 2    Array: ZZZZZ01p-mp HPE Alletra Storage</t>
+          <t>Generated: 2026-06-16 05:27:47    Switches: swd77 Domain 1; swd77 Domain 2    Array: ZZZZZ01p-mp HPE Alletra Storage</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O22"/>
+  <dimension ref="A1:P22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2957,8 +2957,9 @@
     <col width="60" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="36" customWidth="1" min="14" max="14"/>
-    <col width="34" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="36" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -3029,10 +3030,15 @@
       </c>
       <c r="N1" s="9" t="inlineStr">
         <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="O1" s="9" t="inlineStr">
+        <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="O1" s="9" t="inlineStr">
+      <c r="P1" s="9" t="inlineStr">
         <is>
           <t>Vuln</t>
         </is>
@@ -3099,15 +3105,20 @@
       </c>
       <c r="M2" s="20" t="inlineStr">
         <is>
-          <t>Brocade01 2026-06-01.log: swd77 (Domain 1)</t>
+          <t>swd77 (Domain 1)</t>
         </is>
       </c>
       <c r="N2" s="20" t="inlineStr">
         <is>
+          <t>Brocade01 2026-06-01.log</t>
+        </is>
+      </c>
+      <c r="O2" s="20" t="inlineStr">
+        <is>
           <t>auth.policy: 0 (off) (22)</t>
         </is>
       </c>
-      <c r="O2" s="20" t="inlineStr">
+      <c r="P2" s="20" t="inlineStr">
         <is>
           <t>SAN - FC Authentication Policy Disabled</t>
         </is>
@@ -3174,15 +3185,20 @@
       </c>
       <c r="M3" s="21" t="inlineStr">
         <is>
-          <t>Brocade01 2026-06-01.log: swd77 (Domain 1)</t>
+          <t>swd77 (Domain 1)</t>
         </is>
       </c>
       <c r="N3" s="21" t="inlineStr">
         <is>
+          <t>Brocade01 2026-06-01.log</t>
+        </is>
+      </c>
+      <c r="O3" s="21" t="inlineStr">
+        <is>
           <t>defzone: allaccess (359)</t>
         </is>
       </c>
-      <c r="O3" s="21" t="inlineStr">
+      <c r="P3" s="21" t="inlineStr">
         <is>
           <t>SAN - Default Zone Allows All Access</t>
         </is>
@@ -3249,15 +3265,20 @@
       </c>
       <c r="M4" s="20" t="inlineStr">
         <is>
-          <t>Brocade02 2026-06-01.log: swd77 (Domain 2)</t>
+          <t>swd77 (Domain 2)</t>
         </is>
       </c>
       <c r="N4" s="20" t="inlineStr">
         <is>
+          <t>Brocade02 2026-06-01.log</t>
+        </is>
+      </c>
+      <c r="O4" s="20" t="inlineStr">
+        <is>
           <t>auth.policy: 0 (off) (22)</t>
         </is>
       </c>
-      <c r="O4" s="20" t="inlineStr">
+      <c r="P4" s="20" t="inlineStr">
         <is>
           <t>SAN - FC Authentication Policy Disabled</t>
         </is>
@@ -3324,15 +3345,20 @@
       </c>
       <c r="M5" s="21" t="inlineStr">
         <is>
-          <t>Brocade02 2026-06-01.log: swd77 (Domain 2)</t>
+          <t>swd77 (Domain 2)</t>
         </is>
       </c>
       <c r="N5" s="21" t="inlineStr">
         <is>
+          <t>Brocade02 2026-06-01.log</t>
+        </is>
+      </c>
+      <c r="O5" s="21" t="inlineStr">
+        <is>
           <t>defzone: allaccess (357)</t>
         </is>
       </c>
-      <c r="O5" s="21" t="inlineStr">
+      <c r="P5" s="21" t="inlineStr">
         <is>
           <t>SAN - Default Zone Allows All Access</t>
         </is>
@@ -3395,15 +3421,20 @@
       </c>
       <c r="M6" s="20" t="inlineStr">
         <is>
-          <t>Alletra 2026-06-09-01.log: ZZZZZ01p-mp</t>
+          <t>ZZZZZ01p-mp</t>
         </is>
       </c>
       <c r="N6" s="20" t="inlineStr">
         <is>
+          <t>Alletra 2026-06-09-01.log</t>
+        </is>
+      </c>
+      <c r="O6" s="20" t="inlineStr">
+        <is>
           <t>5 host(s) without CHAP</t>
         </is>
       </c>
-      <c r="O6" s="20" t="inlineStr">
+      <c r="P6" s="20" t="inlineStr">
         <is>
           <t>SAN - No CHAP on Storage Hosts</t>
         </is>
@@ -3466,15 +3497,20 @@
       </c>
       <c r="M7" s="21" t="inlineStr">
         <is>
-          <t>Alletra 2026-06-09-01.log: ZZZZZ01p-mp</t>
+          <t>ZZZZZ01p-mp</t>
         </is>
       </c>
       <c r="N7" s="21" t="inlineStr">
         <is>
+          <t>Alletra 2026-06-09-01.log</t>
+        </is>
+      </c>
+      <c r="O7" s="21" t="inlineStr">
+        <is>
           <t>commands: showpasswordpolicy, showsnmp, showsyslog, showaudit, showtime</t>
         </is>
       </c>
-      <c r="O7" s="21" t="inlineStr">
+      <c r="P7" s="21" t="inlineStr">
         <is>
           <t>SAN - Security Baseline Not Verifiable</t>
         </is>
@@ -3537,15 +3573,20 @@
       </c>
       <c r="M8" s="20" t="inlineStr">
         <is>
-          <t>Alletra 2026-06-09-01.log: ZZZZZ01p-mp</t>
+          <t>ZZZZZ01p-mp</t>
         </is>
       </c>
       <c r="N8" s="20" t="inlineStr">
         <is>
+          <t>Alletra 2026-06-09-01.log</t>
+        </is>
+      </c>
+      <c r="O8" s="20" t="inlineStr">
+        <is>
           <t>showsshkey: No SSH key found</t>
         </is>
       </c>
-      <c r="O8" s="20" t="inlineStr">
+      <c r="P8" s="20" t="inlineStr">
         <is>
           <t>SAN - No SSH Keys Configured</t>
         </is>
@@ -3604,15 +3645,20 @@
       </c>
       <c r="M9" s="21" t="inlineStr">
         <is>
-          <t>Volumes_Inventory_06092026_120519.csv: hai01p-mp</t>
+          <t>hai01p-mp</t>
         </is>
       </c>
       <c r="N9" s="21" t="inlineStr">
         <is>
+          <t>Volumes_Inventory_06092026_120519.csv</t>
+        </is>
+      </c>
+      <c r="O9" s="21" t="inlineStr">
+        <is>
           <t>Volume Set: DevTest1</t>
         </is>
       </c>
-      <c r="O9" s="21" t="inlineStr">
+      <c r="P9" s="21" t="inlineStr">
         <is>
           <t>SAN - No Volume Replication Configured</t>
         </is>
@@ -3671,15 +3717,20 @@
       </c>
       <c r="M10" s="20" t="inlineStr">
         <is>
-          <t>Volumes_Inventory_06092026_120519.csv: hai01p-mp</t>
+          <t>hai01p-mp</t>
         </is>
       </c>
       <c r="N10" s="20" t="inlineStr">
         <is>
+          <t>Volumes_Inventory_06092026_120519.csv</t>
+        </is>
+      </c>
+      <c r="O10" s="20" t="inlineStr">
+        <is>
           <t>Volume Set: Infrastructure1</t>
         </is>
       </c>
-      <c r="O10" s="20" t="inlineStr">
+      <c r="P10" s="20" t="inlineStr">
         <is>
           <t>SAN - No Volume Replication Configured</t>
         </is>
@@ -3738,15 +3789,20 @@
       </c>
       <c r="M11" s="21" t="inlineStr">
         <is>
-          <t>Volumes_Inventory_06092026_120519.csv: hai01p-mp</t>
+          <t>hai01p-mp</t>
         </is>
       </c>
       <c r="N11" s="21" t="inlineStr">
         <is>
+          <t>Volumes_Inventory_06092026_120519.csv</t>
+        </is>
+      </c>
+      <c r="O11" s="21" t="inlineStr">
+        <is>
           <t>Volume Set: Infrastructure2</t>
         </is>
       </c>
-      <c r="O11" s="21" t="inlineStr">
+      <c r="P11" s="21" t="inlineStr">
         <is>
           <t>SAN - No Volume Replication Configured</t>
         </is>
@@ -3805,15 +3861,20 @@
       </c>
       <c r="M12" s="20" t="inlineStr">
         <is>
-          <t>Volumes_Inventory_06092026_120519.csv: hai01p-mp</t>
+          <t>hai01p-mp</t>
         </is>
       </c>
       <c r="N12" s="20" t="inlineStr">
         <is>
+          <t>Volumes_Inventory_06092026_120519.csv</t>
+        </is>
+      </c>
+      <c r="O12" s="20" t="inlineStr">
+        <is>
           <t>Volume Set: Production1</t>
         </is>
       </c>
-      <c r="O12" s="20" t="inlineStr">
+      <c r="P12" s="20" t="inlineStr">
         <is>
           <t>SAN - No Volume Replication Configured</t>
         </is>
@@ -3872,15 +3933,20 @@
       </c>
       <c r="M13" s="21" t="inlineStr">
         <is>
-          <t>Volumes_Inventory_06092026_120519.csv: hai01p-mp</t>
+          <t>hai01p-mp</t>
         </is>
       </c>
       <c r="N13" s="21" t="inlineStr">
         <is>
+          <t>Volumes_Inventory_06092026_120519.csv</t>
+        </is>
+      </c>
+      <c r="O13" s="21" t="inlineStr">
+        <is>
           <t>Volume Set: Production2</t>
         </is>
       </c>
-      <c r="O13" s="21" t="inlineStr">
+      <c r="P13" s="21" t="inlineStr">
         <is>
           <t>SAN - No Volume Replication Configured</t>
         </is>
@@ -3947,15 +4013,20 @@
       </c>
       <c r="M14" s="20" t="inlineStr">
         <is>
-          <t>Brocade01 2026-06-01.log: swd77 (Domain 1)</t>
+          <t>swd77 (Domain 1)</t>
         </is>
       </c>
       <c r="N14" s="20" t="inlineStr">
         <is>
+          <t>Brocade01 2026-06-01.log</t>
+        </is>
+      </c>
+      <c r="O14" s="20" t="inlineStr">
+        <is>
           <t>[Banner] section empty (377)</t>
         </is>
       </c>
-      <c r="O14" s="20" t="inlineStr">
+      <c r="P14" s="20" t="inlineStr">
         <is>
           <t>SAN - No Login Banner Configured</t>
         </is>
@@ -4018,15 +4089,20 @@
       </c>
       <c r="M15" s="21" t="inlineStr">
         <is>
-          <t>Brocade01 2026-06-01.log: swd77 (Domain 1)</t>
+          <t>swd77 (Domain 1)</t>
         </is>
       </c>
       <c r="N15" s="21" t="inlineStr">
         <is>
+          <t>Brocade01 2026-06-01.log</t>
+        </is>
+      </c>
+      <c r="O15" s="21" t="inlineStr">
+        <is>
           <t>4 orphaned zone(s) (419)</t>
         </is>
       </c>
-      <c r="O15" s="21" t="inlineStr">
+      <c r="P15" s="21" t="inlineStr">
         <is>
           <t>SAN - Stale Zone Definitions</t>
         </is>
@@ -4093,15 +4169,20 @@
       </c>
       <c r="M16" s="20" t="inlineStr">
         <is>
-          <t>Brocade02 2026-06-01.log: swd77 (Domain 2)</t>
+          <t>swd77 (Domain 2)</t>
         </is>
       </c>
       <c r="N16" s="20" t="inlineStr">
         <is>
+          <t>Brocade02 2026-06-01.log</t>
+        </is>
+      </c>
+      <c r="O16" s="20" t="inlineStr">
+        <is>
           <t>[Banner] section empty (375)</t>
         </is>
       </c>
-      <c r="O16" s="20" t="inlineStr">
+      <c r="P16" s="20" t="inlineStr">
         <is>
           <t>SAN - No Login Banner Configured</t>
         </is>
@@ -4164,15 +4245,20 @@
       </c>
       <c r="M17" s="21" t="inlineStr">
         <is>
-          <t>Brocade02 2026-06-01.log: swd77 (Domain 2)</t>
+          <t>swd77 (Domain 2)</t>
         </is>
       </c>
       <c r="N17" s="21" t="inlineStr">
         <is>
+          <t>Brocade02 2026-06-01.log</t>
+        </is>
+      </c>
+      <c r="O17" s="21" t="inlineStr">
+        <is>
           <t>5 orphaned zone(s) (417)</t>
         </is>
       </c>
-      <c r="O17" s="21" t="inlineStr">
+      <c r="P17" s="21" t="inlineStr">
         <is>
           <t>SAN - Stale Zone Definitions</t>
         </is>
@@ -4231,15 +4317,20 @@
       </c>
       <c r="M18" s="20" t="inlineStr">
         <is>
-          <t>Alletra 2026-06-09-01.log: ZZZZZ01p-mp</t>
+          <t>ZZZZZ01p-mp</t>
         </is>
       </c>
       <c r="N18" s="20" t="inlineStr">
         <is>
+          <t>Alletra 2026-06-09-01.log</t>
+        </is>
+      </c>
+      <c r="O18" s="20" t="inlineStr">
+        <is>
           <t>loss_sync: 0:3:2, 0:3:4, 1:3:2, 1:3:4</t>
         </is>
       </c>
-      <c r="O18" s="20" t="inlineStr">
+      <c r="P18" s="20" t="inlineStr">
         <is>
           <t>SAN - Degraded FC Ports</t>
         </is>
@@ -4302,15 +4393,20 @@
       </c>
       <c r="M19" s="21" t="inlineStr">
         <is>
-          <t>Alletra 2026-06-09-01.log: ZZZZZ01p-mp</t>
+          <t>ZZZZZ01p-mp</t>
         </is>
       </c>
       <c r="N19" s="21" t="inlineStr">
         <is>
+          <t>Alletra 2026-06-09-01.log</t>
+        </is>
+      </c>
+      <c r="O19" s="21" t="inlineStr">
+        <is>
           <t>WSAPI: Enabled / Active on HTTPS 443</t>
         </is>
       </c>
-      <c r="O19" s="21" t="inlineStr">
+      <c r="P19" s="21" t="inlineStr">
         <is>
           <t>SAN - REST API Exposed</t>
         </is>
@@ -4365,15 +4461,20 @@
       </c>
       <c r="M20" s="20" t="inlineStr">
         <is>
-          <t>Brocade01 2026-06-01.log: swd77 (Domain 1)</t>
+          <t>swd77 (Domain 1)</t>
         </is>
       </c>
       <c r="N20" s="20" t="inlineStr">
         <is>
+          <t>Brocade01 2026-06-01.log</t>
+        </is>
+      </c>
+      <c r="O20" s="20" t="inlineStr">
+        <is>
           <t>maps.activePolicy: dflt_base_policy</t>
         </is>
       </c>
-      <c r="O20" s="20" t="inlineStr">
+      <c r="P20" s="20" t="inlineStr">
         <is>
           <t>SAN - Default MAPS Monitoring Policy</t>
         </is>
@@ -4428,15 +4529,20 @@
       </c>
       <c r="M21" s="21" t="inlineStr">
         <is>
-          <t>Brocade02 2026-06-01.log: swd77 (Domain 2)</t>
+          <t>swd77 (Domain 2)</t>
         </is>
       </c>
       <c r="N21" s="21" t="inlineStr">
         <is>
+          <t>Brocade02 2026-06-01.log</t>
+        </is>
+      </c>
+      <c r="O21" s="21" t="inlineStr">
+        <is>
           <t>maps.activePolicy: dflt_base_policy</t>
         </is>
       </c>
-      <c r="O21" s="21" t="inlineStr">
+      <c r="P21" s="21" t="inlineStr">
         <is>
           <t>SAN - Default MAPS Monitoring Policy</t>
         </is>
@@ -4495,22 +4601,27 @@
       </c>
       <c r="M22" s="20" t="inlineStr">
         <is>
-          <t>storage-devices-export-data.csv: VMware ESXi</t>
+          <t>VMware ESXi</t>
         </is>
       </c>
       <c r="N22" s="20" t="inlineStr">
         <is>
+          <t>storage-devices-export-data.csv</t>
+        </is>
+      </c>
+      <c r="O22" s="20" t="inlineStr">
+        <is>
           <t>5 FC disk(s)</t>
         </is>
       </c>
-      <c r="O22" s="20" t="inlineStr">
+      <c r="P22" s="20" t="inlineStr">
         <is>
           <t>SAN - Perennially Reserved Not Configured</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O1"/>
+  <autoFilter ref="A1:P1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>